<commit_message>
download SP2D tgl 1 di SAKTI
dowload SP2D yang kurang dari SAKTI
</commit_message>
<xml_diff>
--- a/Database/SP2D.xlsx
+++ b/Database/SP2D.xlsx
@@ -601,7 +601,7 @@
       <c r="A3" s="4" t="inlineStr">
         <is>
           <r>
-            <t xml:space="preserve">Periode Juli 2025</t>
+            <t xml:space="preserve">Periode Agustus 2025</t>
           </r>
         </is>
       </c>
@@ -979,22 +979,22 @@
       <c r="U9" s="10" t="inlineStr"/>
       <c r="V9" s="10" t="inlineStr"/>
       <c r="W9" s="11" t="n">
-        <v>5.0261287724E10</v>
+        <v>5.7092109652E10</v>
       </c>
       <c r="X9" s="11" t="n">
-        <v>6.830821928E9</v>
+        <v>3.331178713E9</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>5.7092109652E10</v>
+        <v>6.0423288365E10</v>
       </c>
       <c r="Z9" s="10" t="inlineStr"/>
       <c r="AA9" s="10" t="inlineStr"/>
       <c r="AB9" s="10" t="inlineStr"/>
       <c r="AC9" s="12" t="n">
-        <v>0.6715865472622302</v>
+        <v>0.7107719062166219</v>
       </c>
       <c r="AD9" s="10" t="n">
-        <v>2.7918690348E10</v>
+        <v>2.4587511635E10</v>
       </c>
       <c r="AE9" s="10" t="inlineStr"/>
       <c r="AF9" s="10" t="inlineStr"/>
@@ -1042,23 +1042,23 @@
       <c r="U10" s="14" t="inlineStr"/>
       <c r="V10" s="14" t="inlineStr"/>
       <c r="W10" s="14" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X10" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y10" s="14" t="inlineStr"/>
       <c r="Z10" s="14" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA10" s="14" t="inlineStr"/>
       <c r="AB10" s="14" t="inlineStr"/>
       <c r="AC10" s="15" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD10" s="15" t="inlineStr"/>
       <c r="AE10" s="14" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF10" s="14" t="inlineStr"/>
       <c r="AG10" s="14" t="inlineStr"/>
@@ -1105,23 +1105,23 @@
       <c r="U11" s="14" t="inlineStr"/>
       <c r="V11" s="14" t="inlineStr"/>
       <c r="W11" s="14" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X11" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y11" s="14" t="inlineStr"/>
       <c r="Z11" s="14" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA11" s="14" t="inlineStr"/>
       <c r="AB11" s="14" t="inlineStr"/>
       <c r="AC11" s="15" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD11" s="15" t="inlineStr"/>
       <c r="AE11" s="14" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF11" s="14" t="inlineStr"/>
       <c r="AG11" s="14" t="inlineStr"/>
@@ -1717,23 +1717,23 @@
       <c r="U21" s="17" t="inlineStr"/>
       <c r="V21" s="17" t="inlineStr"/>
       <c r="W21" s="17" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X21" s="17" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y21" s="17" t="inlineStr"/>
       <c r="Z21" s="17" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA21" s="17" t="inlineStr"/>
       <c r="AB21" s="17" t="inlineStr"/>
       <c r="AC21" s="18" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD21" s="18" t="inlineStr"/>
       <c r="AE21" s="17" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF21" s="17" t="inlineStr"/>
       <c r="AG21" s="17" t="inlineStr"/>
@@ -1780,23 +1780,23 @@
       <c r="U22" s="21" t="inlineStr"/>
       <c r="V22" s="21" t="inlineStr"/>
       <c r="W22" s="22" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X22" s="22" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y22" s="22" t="inlineStr"/>
       <c r="Z22" s="21" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA22" s="21" t="inlineStr"/>
       <c r="AB22" s="21" t="inlineStr"/>
       <c r="AC22" s="23" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD22" s="23" t="inlineStr"/>
       <c r="AE22" s="21" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF22" s="21" t="inlineStr"/>
       <c r="AG22" s="21" t="inlineStr"/>
@@ -1843,23 +1843,23 @@
       <c r="U23" s="25" t="inlineStr"/>
       <c r="V23" s="25" t="inlineStr"/>
       <c r="W23" s="25" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X23" s="25" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y23" s="25" t="inlineStr"/>
       <c r="Z23" s="25" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA23" s="25" t="inlineStr"/>
       <c r="AB23" s="25" t="inlineStr"/>
       <c r="AC23" s="26" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD23" s="26" t="inlineStr"/>
       <c r="AE23" s="25" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF23" s="25" t="inlineStr"/>
       <c r="AG23" s="25" t="inlineStr"/>
@@ -1906,23 +1906,23 @@
       <c r="U24" s="14" t="inlineStr"/>
       <c r="V24" s="14" t="inlineStr"/>
       <c r="W24" s="14" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X24" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y24" s="14" t="inlineStr"/>
       <c r="Z24" s="14" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA24" s="14" t="inlineStr"/>
       <c r="AB24" s="14" t="inlineStr"/>
       <c r="AC24" s="15" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD24" s="15" t="inlineStr"/>
       <c r="AE24" s="14" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF24" s="14" t="inlineStr"/>
       <c r="AG24" s="14" t="inlineStr"/>
@@ -1969,23 +1969,23 @@
       <c r="U25" s="14" t="inlineStr"/>
       <c r="V25" s="14" t="inlineStr"/>
       <c r="W25" s="14" t="n">
-        <v>3.02705832E9</v>
+        <v>3.53156804E9</v>
       </c>
       <c r="X25" s="14" t="n">
-        <v>5.0450972E8</v>
+        <v>5.018E8</v>
       </c>
       <c r="Y25" s="14" t="inlineStr"/>
       <c r="Z25" s="14" t="n">
-        <v>3.53156804E9</v>
+        <v>4.03336804E9</v>
       </c>
       <c r="AA25" s="14" t="inlineStr"/>
       <c r="AB25" s="14" t="inlineStr"/>
       <c r="AC25" s="15" t="n">
-        <v>0.699883637049697</v>
+        <v>0.7993300033928294</v>
       </c>
       <c r="AD25" s="15" t="inlineStr"/>
       <c r="AE25" s="14" t="n">
-        <v>1.51436796E9</v>
+        <v>1.01256796E9</v>
       </c>
       <c r="AF25" s="14" t="inlineStr"/>
       <c r="AG25" s="14" t="inlineStr"/>
@@ -2026,23 +2026,23 @@
       <c r="U26" s="14" t="inlineStr"/>
       <c r="V26" s="14" t="inlineStr"/>
       <c r="W26" s="14" t="n">
-        <v>2.592E8</v>
+        <v>3.024E8</v>
       </c>
       <c r="X26" s="14" t="n">
         <v>4.32E7</v>
       </c>
       <c r="Y26" s="14" t="inlineStr"/>
       <c r="Z26" s="14" t="n">
-        <v>3.024E8</v>
+        <v>3.456E8</v>
       </c>
       <c r="AA26" s="14" t="inlineStr"/>
       <c r="AB26" s="14" t="inlineStr"/>
       <c r="AC26" s="15" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="AD26" s="15" t="inlineStr"/>
       <c r="AE26" s="14" t="n">
-        <v>1.296E8</v>
+        <v>8.64E7</v>
       </c>
       <c r="AF26" s="14" t="inlineStr"/>
       <c r="AG26" s="14" t="inlineStr"/>
@@ -2083,23 +2083,23 @@
       <c r="U27" s="14" t="inlineStr"/>
       <c r="V27" s="14" t="inlineStr"/>
       <c r="W27" s="14" t="n">
-        <v>2.6676E9</v>
+        <v>3.1122E9</v>
       </c>
       <c r="X27" s="14" t="n">
         <v>4.446E8</v>
       </c>
       <c r="Y27" s="14" t="inlineStr"/>
       <c r="Z27" s="14" t="n">
-        <v>3.1122E9</v>
+        <v>3.5568E9</v>
       </c>
       <c r="AA27" s="14" t="inlineStr"/>
       <c r="AB27" s="14" t="inlineStr"/>
       <c r="AC27" s="15" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="AD27" s="15" t="inlineStr"/>
       <c r="AE27" s="14" t="n">
-        <v>1.3338E9</v>
+        <v>8.892E8</v>
       </c>
       <c r="AF27" s="14" t="inlineStr"/>
       <c r="AG27" s="14" t="inlineStr"/>
@@ -2140,23 +2140,23 @@
       <c r="U28" s="14" t="inlineStr"/>
       <c r="V28" s="14" t="inlineStr"/>
       <c r="W28" s="14" t="n">
-        <v>8.4E7</v>
+        <v>9.8E7</v>
       </c>
       <c r="X28" s="14" t="n">
         <v>1.4E7</v>
       </c>
       <c r="Y28" s="14" t="inlineStr"/>
       <c r="Z28" s="14" t="n">
-        <v>9.8E7</v>
+        <v>1.12E8</v>
       </c>
       <c r="AA28" s="14" t="inlineStr"/>
       <c r="AB28" s="14" t="inlineStr"/>
       <c r="AC28" s="15" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="AD28" s="15" t="inlineStr"/>
       <c r="AE28" s="14" t="n">
-        <v>4.2E7</v>
+        <v>2.8E7</v>
       </c>
       <c r="AF28" s="14" t="inlineStr"/>
       <c r="AG28" s="14" t="inlineStr"/>
@@ -2197,10 +2197,10 @@
       <c r="U29" s="14" t="inlineStr"/>
       <c r="V29" s="14" t="inlineStr"/>
       <c r="W29" s="14" t="n">
-        <v>1.625832E7</v>
+        <v>1.896804E7</v>
       </c>
       <c r="X29" s="14" t="n">
-        <v>2709720.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y29" s="14" t="inlineStr"/>
       <c r="Z29" s="14" t="n">
@@ -2443,23 +2443,23 @@
       <c r="U33" s="14" t="inlineStr"/>
       <c r="V33" s="14" t="inlineStr"/>
       <c r="W33" s="14" t="n">
-        <v>4.7234229404E10</v>
+        <v>5.3560541612E10</v>
       </c>
       <c r="X33" s="14" t="n">
-        <v>6.326312208E9</v>
+        <v>2.829378713E9</v>
       </c>
       <c r="Y33" s="14" t="inlineStr"/>
       <c r="Z33" s="14" t="n">
-        <v>5.3560541612E10</v>
+        <v>5.6389920325E10</v>
       </c>
       <c r="AA33" s="14" t="inlineStr"/>
       <c r="AB33" s="14" t="inlineStr"/>
       <c r="AC33" s="15" t="n">
-        <v>0.6698009467258019</v>
+        <v>0.7051837207526546</v>
       </c>
       <c r="AD33" s="15" t="inlineStr"/>
       <c r="AE33" s="14" t="n">
-        <v>2.6404322388E10</v>
+        <v>2.3574943675E10</v>
       </c>
       <c r="AF33" s="14" t="inlineStr"/>
       <c r="AG33" s="14" t="inlineStr"/>
@@ -2550,23 +2550,23 @@
       <c r="U35" s="14" t="inlineStr"/>
       <c r="V35" s="14" t="inlineStr"/>
       <c r="W35" s="14" t="n">
-        <v>4.7234229404E10</v>
+        <v>5.3560541612E10</v>
       </c>
       <c r="X35" s="14" t="n">
-        <v>6.326312208E9</v>
+        <v>2.829378713E9</v>
       </c>
       <c r="Y35" s="14" t="inlineStr"/>
       <c r="Z35" s="14" t="n">
-        <v>5.3560541612E10</v>
+        <v>5.6389920325E10</v>
       </c>
       <c r="AA35" s="14" t="inlineStr"/>
       <c r="AB35" s="14" t="inlineStr"/>
       <c r="AC35" s="15" t="n">
-        <v>0.6698009467258019</v>
+        <v>0.7051837207526546</v>
       </c>
       <c r="AD35" s="15" t="inlineStr"/>
       <c r="AE35" s="14" t="n">
-        <v>2.6404322388E10</v>
+        <v>2.3574943675E10</v>
       </c>
       <c r="AF35" s="14" t="inlineStr"/>
       <c r="AG35" s="14" t="inlineStr"/>
@@ -2613,23 +2613,23 @@
       <c r="U36" s="17" t="inlineStr"/>
       <c r="V36" s="17" t="inlineStr"/>
       <c r="W36" s="17" t="n">
-        <v>4.7233629404E10</v>
+        <v>5.3559941612E10</v>
       </c>
       <c r="X36" s="17" t="n">
-        <v>6.326312208E9</v>
+        <v>2.829378713E9</v>
       </c>
       <c r="Y36" s="17" t="inlineStr"/>
       <c r="Z36" s="17" t="n">
-        <v>5.3559941612E10</v>
+        <v>5.6389320325E10</v>
       </c>
       <c r="AA36" s="17" t="inlineStr"/>
       <c r="AB36" s="17" t="inlineStr"/>
       <c r="AC36" s="18" t="n">
-        <v>0.6697984691261587</v>
+        <v>0.7051815086424106</v>
       </c>
       <c r="AD36" s="18" t="inlineStr"/>
       <c r="AE36" s="17" t="n">
-        <v>2.6404322388E10</v>
+        <v>2.3574943675E10</v>
       </c>
       <c r="AF36" s="17" t="inlineStr"/>
       <c r="AG36" s="17" t="inlineStr"/>
@@ -3837,10 +3837,10 @@
       <c r="U56" s="21" t="inlineStr"/>
       <c r="V56" s="21" t="inlineStr"/>
       <c r="W56" s="22" t="n">
-        <v>3949100.0</v>
+        <v>9686100.0</v>
       </c>
       <c r="X56" s="22" t="n">
-        <v>5737000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y56" s="22" t="inlineStr"/>
       <c r="Z56" s="21" t="n">
@@ -3900,10 +3900,10 @@
       <c r="U57" s="25" t="inlineStr"/>
       <c r="V57" s="25" t="inlineStr"/>
       <c r="W57" s="25" t="n">
-        <v>3949100.0</v>
+        <v>9686100.0</v>
       </c>
       <c r="X57" s="25" t="n">
-        <v>5737000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y57" s="25" t="inlineStr"/>
       <c r="Z57" s="25" t="n">
@@ -3963,10 +3963,10 @@
       <c r="U58" s="14" t="inlineStr"/>
       <c r="V58" s="14" t="inlineStr"/>
       <c r="W58" s="14" t="n">
-        <v>600000.0</v>
+        <v>2400000.0</v>
       </c>
       <c r="X58" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y58" s="14" t="inlineStr"/>
       <c r="Z58" s="14" t="n">
@@ -4026,10 +4026,10 @@
       <c r="U59" s="14" t="inlineStr"/>
       <c r="V59" s="14" t="inlineStr"/>
       <c r="W59" s="14" t="n">
-        <v>0.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="X59" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y59" s="14" t="inlineStr"/>
       <c r="Z59" s="14" t="n">
@@ -4127,10 +4127,10 @@
       <c r="U61" s="14" t="inlineStr"/>
       <c r="V61" s="14" t="inlineStr"/>
       <c r="W61" s="14" t="n">
-        <v>0.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="X61" s="14" t="n">
-        <v>1800000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y61" s="14" t="inlineStr"/>
       <c r="Z61" s="14" t="n">
@@ -4310,10 +4310,10 @@
       <c r="U64" s="14" t="inlineStr"/>
       <c r="V64" s="14" t="inlineStr"/>
       <c r="W64" s="14" t="n">
-        <v>3349100.0</v>
+        <v>7286100.0</v>
       </c>
       <c r="X64" s="14" t="n">
-        <v>3937000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y64" s="14" t="inlineStr"/>
       <c r="Z64" s="14" t="n">
@@ -4373,10 +4373,10 @@
       <c r="U65" s="14" t="inlineStr"/>
       <c r="V65" s="14" t="inlineStr"/>
       <c r="W65" s="14" t="n">
-        <v>3349100.0</v>
+        <v>7286100.0</v>
       </c>
       <c r="X65" s="14" t="n">
-        <v>3937000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y65" s="14" t="inlineStr"/>
       <c r="Z65" s="14" t="n">
@@ -4430,10 +4430,10 @@
       <c r="U66" s="14" t="inlineStr"/>
       <c r="V66" s="14" t="inlineStr"/>
       <c r="W66" s="14" t="n">
-        <v>2600000.0</v>
+        <v>6537000.0</v>
       </c>
       <c r="X66" s="14" t="n">
-        <v>3937000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y66" s="14" t="inlineStr"/>
       <c r="Z66" s="14" t="n">
@@ -4733,23 +4733,23 @@
       <c r="U71" s="21" t="inlineStr"/>
       <c r="V71" s="21" t="inlineStr"/>
       <c r="W71" s="22" t="n">
-        <v>4.7228630304E10</v>
+        <v>5.3549205512E10</v>
       </c>
       <c r="X71" s="22" t="n">
-        <v>6.320575208E9</v>
+        <v>2.829378713E9</v>
       </c>
       <c r="Y71" s="22" t="inlineStr"/>
       <c r="Z71" s="21" t="n">
-        <v>5.3549205512E10</v>
+        <v>5.6378584225E10</v>
       </c>
       <c r="AA71" s="21" t="inlineStr"/>
       <c r="AB71" s="21" t="inlineStr"/>
       <c r="AC71" s="23" t="n">
-        <v>0.6698194241608939</v>
+        <v>0.7052106648367253</v>
       </c>
       <c r="AD71" s="23" t="inlineStr"/>
       <c r="AE71" s="21" t="n">
-        <v>2.6396528488E10</v>
+        <v>2.3567149775E10</v>
       </c>
       <c r="AF71" s="21" t="inlineStr"/>
       <c r="AG71" s="21" t="inlineStr"/>
@@ -4796,23 +4796,23 @@
       <c r="U72" s="25" t="inlineStr"/>
       <c r="V72" s="25" t="inlineStr"/>
       <c r="W72" s="25" t="n">
-        <v>4.4677440659E10</v>
+        <v>5.0573817532E10</v>
       </c>
       <c r="X72" s="25" t="n">
-        <v>5.896376873E9</v>
+        <v>2.755968713E9</v>
       </c>
       <c r="Y72" s="25" t="inlineStr"/>
       <c r="Z72" s="25" t="n">
-        <v>5.0573817532E10</v>
+        <v>5.3329786245E10</v>
       </c>
       <c r="AA72" s="25" t="inlineStr"/>
       <c r="AB72" s="25" t="inlineStr"/>
       <c r="AC72" s="26" t="n">
-        <v>0.6807624358417722</v>
+        <v>0.7178598919113772</v>
       </c>
       <c r="AD72" s="26" t="inlineStr"/>
       <c r="AE72" s="25" t="n">
-        <v>2.3716147468E10</v>
+        <v>2.0960178755E10</v>
       </c>
       <c r="AF72" s="25" t="inlineStr"/>
       <c r="AG72" s="25" t="inlineStr"/>
@@ -4859,23 +4859,23 @@
       <c r="U73" s="14" t="inlineStr"/>
       <c r="V73" s="14" t="inlineStr"/>
       <c r="W73" s="14" t="n">
-        <v>3.39277532E9</v>
+        <v>3.798075364E9</v>
       </c>
       <c r="X73" s="14" t="n">
-        <v>4.05300044E8</v>
+        <v>3.8947414E8</v>
       </c>
       <c r="Y73" s="14" t="inlineStr"/>
       <c r="Z73" s="14" t="n">
-        <v>3.798075364E9</v>
+        <v>4.187549504E9</v>
       </c>
       <c r="AA73" s="14" t="inlineStr"/>
       <c r="AB73" s="14" t="inlineStr"/>
       <c r="AC73" s="15" t="n">
-        <v>0.592813113053055</v>
+        <v>0.6536032120530656</v>
       </c>
       <c r="AD73" s="15" t="inlineStr"/>
       <c r="AE73" s="14" t="n">
-        <v>2.608792636E9</v>
+        <v>2.219318496E9</v>
       </c>
       <c r="AF73" s="14" t="inlineStr"/>
       <c r="AG73" s="14" t="inlineStr"/>
@@ -4922,23 +4922,23 @@
       <c r="U74" s="14" t="inlineStr"/>
       <c r="V74" s="14" t="inlineStr"/>
       <c r="W74" s="14" t="n">
-        <v>1.3295234E9</v>
+        <v>1.4858101E9</v>
       </c>
       <c r="X74" s="14" t="n">
-        <v>1.562867E8</v>
+        <v>1.64507E8</v>
       </c>
       <c r="Y74" s="14" t="inlineStr"/>
       <c r="Z74" s="14" t="n">
-        <v>1.4858101E9</v>
+        <v>1.6503171E9</v>
       </c>
       <c r="AA74" s="14" t="inlineStr"/>
       <c r="AB74" s="14" t="inlineStr"/>
       <c r="AC74" s="15" t="n">
-        <v>0.5301905004553227</v>
+        <v>0.5888925167213339</v>
       </c>
       <c r="AD74" s="15" t="inlineStr"/>
       <c r="AE74" s="14" t="n">
-        <v>1.3165979E9</v>
+        <v>1.1520909E9</v>
       </c>
       <c r="AF74" s="14" t="inlineStr"/>
       <c r="AG74" s="14" t="inlineStr"/>
@@ -4979,23 +4979,23 @@
       <c r="U75" s="14" t="inlineStr"/>
       <c r="V75" s="14" t="inlineStr"/>
       <c r="W75" s="14" t="n">
-        <v>9.99343E8</v>
+        <v>1.1556297E9</v>
       </c>
       <c r="X75" s="14" t="n">
-        <v>1.562867E8</v>
+        <v>1.64507E8</v>
       </c>
       <c r="Y75" s="14" t="inlineStr"/>
       <c r="Z75" s="14" t="n">
-        <v>1.1556297E9</v>
+        <v>1.3201367E9</v>
       </c>
       <c r="AA75" s="14" t="inlineStr"/>
       <c r="AB75" s="14" t="inlineStr"/>
       <c r="AC75" s="15" t="n">
-        <v>0.4699974377745242</v>
+        <v>0.5369028387831463</v>
       </c>
       <c r="AD75" s="15" t="inlineStr"/>
       <c r="AE75" s="14" t="n">
-        <v>1.3031703E9</v>
+        <v>1.1386633E9</v>
       </c>
       <c r="AF75" s="14" t="inlineStr"/>
       <c r="AG75" s="14" t="inlineStr"/>
@@ -5156,23 +5156,23 @@
       <c r="U78" s="14" t="inlineStr"/>
       <c r="V78" s="14" t="inlineStr"/>
       <c r="W78" s="14" t="n">
-        <v>16177.0</v>
+        <v>17822.0</v>
       </c>
       <c r="X78" s="14" t="n">
-        <v>1645.0</v>
+        <v>1727.0</v>
       </c>
       <c r="Y78" s="14" t="inlineStr"/>
       <c r="Z78" s="14" t="n">
-        <v>17822.0</v>
+        <v>19549.0</v>
       </c>
       <c r="AA78" s="14" t="inlineStr"/>
       <c r="AB78" s="14" t="inlineStr"/>
       <c r="AC78" s="15" t="n">
-        <v>0.5940666666666666</v>
+        <v>0.6516333333333333</v>
       </c>
       <c r="AD78" s="15" t="inlineStr"/>
       <c r="AE78" s="14" t="n">
-        <v>12178.0</v>
+        <v>10451.0</v>
       </c>
       <c r="AF78" s="14" t="inlineStr"/>
       <c r="AG78" s="14" t="inlineStr"/>
@@ -5213,23 +5213,23 @@
       <c r="U79" s="14" t="inlineStr"/>
       <c r="V79" s="14" t="inlineStr"/>
       <c r="W79" s="14" t="n">
-        <v>11595.0</v>
+        <v>13240.0</v>
       </c>
       <c r="X79" s="14" t="n">
-        <v>1645.0</v>
+        <v>1727.0</v>
       </c>
       <c r="Y79" s="14" t="inlineStr"/>
       <c r="Z79" s="14" t="n">
-        <v>13240.0</v>
+        <v>14967.0</v>
       </c>
       <c r="AA79" s="14" t="inlineStr"/>
       <c r="AB79" s="14" t="inlineStr"/>
       <c r="AC79" s="15" t="n">
-        <v>0.5516666666666666</v>
+        <v>0.623625</v>
       </c>
       <c r="AD79" s="15" t="inlineStr"/>
       <c r="AE79" s="14" t="n">
-        <v>10760.0</v>
+        <v>9033.0</v>
       </c>
       <c r="AF79" s="14" t="inlineStr"/>
       <c r="AG79" s="14" t="inlineStr"/>
@@ -5390,23 +5390,23 @@
       <c r="U82" s="14" t="inlineStr"/>
       <c r="V82" s="14" t="inlineStr"/>
       <c r="W82" s="14" t="n">
-        <v>1.0164363E8</v>
+        <v>1.1333796E8</v>
       </c>
       <c r="X82" s="14" t="n">
-        <v>1.169433E7</v>
+        <v>1.251636E7</v>
       </c>
       <c r="Y82" s="14" t="inlineStr"/>
       <c r="Z82" s="14" t="n">
-        <v>1.1333796E8</v>
+        <v>1.2585432E8</v>
       </c>
       <c r="AA82" s="14" t="inlineStr"/>
       <c r="AB82" s="14" t="inlineStr"/>
       <c r="AC82" s="15" t="n">
-        <v>0.622736043956044</v>
+        <v>0.6915072527472528</v>
       </c>
       <c r="AD82" s="15" t="inlineStr"/>
       <c r="AE82" s="14" t="n">
-        <v>6.866204E7</v>
+        <v>5.614568E7</v>
       </c>
       <c r="AF82" s="14" t="inlineStr"/>
       <c r="AG82" s="14" t="inlineStr"/>
@@ -5447,23 +5447,23 @@
       <c r="U83" s="14" t="inlineStr"/>
       <c r="V83" s="14" t="inlineStr"/>
       <c r="W83" s="14" t="n">
-        <v>7.644531E7</v>
+        <v>8.813964E7</v>
       </c>
       <c r="X83" s="14" t="n">
-        <v>1.169433E7</v>
+        <v>1.251636E7</v>
       </c>
       <c r="Y83" s="14" t="inlineStr"/>
       <c r="Z83" s="14" t="n">
-        <v>8.813964E7</v>
+        <v>1.00656E8</v>
       </c>
       <c r="AA83" s="14" t="inlineStr"/>
       <c r="AB83" s="14" t="inlineStr"/>
       <c r="AC83" s="15" t="n">
-        <v>0.5649976923076923</v>
+        <v>0.6452307692307693</v>
       </c>
       <c r="AD83" s="15" t="inlineStr"/>
       <c r="AE83" s="14" t="n">
-        <v>6.786036E7</v>
+        <v>5.5344E7</v>
       </c>
       <c r="AF83" s="14" t="inlineStr"/>
       <c r="AG83" s="14" t="inlineStr"/>
@@ -5624,23 +5624,23 @@
       <c r="U86" s="14" t="inlineStr"/>
       <c r="V86" s="14" t="inlineStr"/>
       <c r="W86" s="14" t="n">
-        <v>3.0975352E7</v>
+        <v>3.4441812E7</v>
       </c>
       <c r="X86" s="14" t="n">
-        <v>3466460.0</v>
+        <v>3795272.0</v>
       </c>
       <c r="Y86" s="14" t="inlineStr"/>
       <c r="Z86" s="14" t="n">
-        <v>3.4441812E7</v>
+        <v>3.8237084E7</v>
       </c>
       <c r="AA86" s="14" t="inlineStr"/>
       <c r="AB86" s="14" t="inlineStr"/>
       <c r="AC86" s="15" t="n">
-        <v>0.6150323571428571</v>
+        <v>0.6828050714285714</v>
       </c>
       <c r="AD86" s="15" t="inlineStr"/>
       <c r="AE86" s="14" t="n">
-        <v>2.1558188E7</v>
+        <v>1.7762916E7</v>
       </c>
       <c r="AF86" s="14" t="inlineStr"/>
       <c r="AG86" s="14" t="inlineStr"/>
@@ -5725,23 +5725,23 @@
       <c r="U88" s="14" t="inlineStr"/>
       <c r="V88" s="14" t="inlineStr"/>
       <c r="W88" s="14" t="n">
-        <v>2.3299294E7</v>
+        <v>2.6765754E7</v>
       </c>
       <c r="X88" s="14" t="n">
-        <v>3466460.0</v>
+        <v>3795272.0</v>
       </c>
       <c r="Y88" s="14" t="inlineStr"/>
       <c r="Z88" s="14" t="n">
-        <v>2.6765754E7</v>
+        <v>3.0561026E7</v>
       </c>
       <c r="AA88" s="14" t="inlineStr"/>
       <c r="AB88" s="14" t="inlineStr"/>
       <c r="AC88" s="15" t="n">
-        <v>0.557619875</v>
+        <v>0.6366880416666667</v>
       </c>
       <c r="AD88" s="15" t="inlineStr"/>
       <c r="AE88" s="14" t="n">
-        <v>2.1234246E7</v>
+        <v>1.7438974E7</v>
       </c>
       <c r="AF88" s="14" t="inlineStr"/>
       <c r="AG88" s="14" t="inlineStr"/>
@@ -5902,23 +5902,23 @@
       <c r="U91" s="14" t="inlineStr"/>
       <c r="V91" s="14" t="inlineStr"/>
       <c r="W91" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.62E7</v>
       </c>
       <c r="X91" s="14" t="n">
         <v>1800000.0</v>
       </c>
       <c r="Y91" s="14" t="inlineStr"/>
       <c r="Z91" s="14" t="n">
-        <v>1.62E7</v>
+        <v>1.8E7</v>
       </c>
       <c r="AA91" s="14" t="inlineStr"/>
       <c r="AB91" s="14" t="inlineStr"/>
       <c r="AC91" s="15" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="AD91" s="15" t="inlineStr"/>
       <c r="AE91" s="14" t="n">
-        <v>9000000.0</v>
+        <v>7200000.0</v>
       </c>
       <c r="AF91" s="14" t="inlineStr"/>
       <c r="AG91" s="14" t="inlineStr"/>
@@ -5959,23 +5959,23 @@
       <c r="U92" s="14" t="inlineStr"/>
       <c r="V92" s="14" t="inlineStr"/>
       <c r="W92" s="14" t="n">
-        <v>1.08E7</v>
+        <v>1.26E7</v>
       </c>
       <c r="X92" s="14" t="n">
         <v>1800000.0</v>
       </c>
       <c r="Y92" s="14" t="inlineStr"/>
       <c r="Z92" s="14" t="n">
-        <v>1.26E7</v>
+        <v>1.44E7</v>
       </c>
       <c r="AA92" s="14" t="inlineStr"/>
       <c r="AB92" s="14" t="inlineStr"/>
       <c r="AC92" s="15" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="AD92" s="15" t="inlineStr"/>
       <c r="AE92" s="14" t="n">
-        <v>9000000.0</v>
+        <v>7200000.0</v>
       </c>
       <c r="AF92" s="14" t="inlineStr"/>
       <c r="AG92" s="14" t="inlineStr"/>
@@ -6136,23 +6136,23 @@
       <c r="U95" s="14" t="inlineStr"/>
       <c r="V95" s="14" t="inlineStr"/>
       <c r="W95" s="14" t="n">
-        <v>9.6112E7</v>
+        <v>1.06486E8</v>
       </c>
       <c r="X95" s="14" t="n">
-        <v>1.0374E7</v>
+        <v>1.1474E7</v>
       </c>
       <c r="Y95" s="14" t="inlineStr"/>
       <c r="Z95" s="14" t="n">
-        <v>1.06486E8</v>
+        <v>1.1796E8</v>
       </c>
       <c r="AA95" s="14" t="inlineStr"/>
       <c r="AB95" s="14" t="inlineStr"/>
       <c r="AC95" s="15" t="n">
-        <v>0.7343153074875529</v>
+        <v>0.8134387024701063</v>
       </c>
       <c r="AD95" s="15" t="inlineStr"/>
       <c r="AE95" s="14" t="n">
-        <v>3.8528E7</v>
+        <v>2.7054E7</v>
       </c>
       <c r="AF95" s="14" t="inlineStr"/>
       <c r="AG95" s="14" t="inlineStr"/>
@@ -6193,23 +6193,23 @@
       <c r="U96" s="14" t="inlineStr"/>
       <c r="V96" s="14" t="inlineStr"/>
       <c r="W96" s="14" t="n">
-        <v>7.2084E7</v>
+        <v>8.2458E7</v>
       </c>
       <c r="X96" s="14" t="n">
-        <v>1.0374E7</v>
+        <v>1.1474E7</v>
       </c>
       <c r="Y96" s="14" t="inlineStr"/>
       <c r="Z96" s="14" t="n">
-        <v>8.2458E7</v>
+        <v>9.3932E7</v>
       </c>
       <c r="AA96" s="14" t="inlineStr"/>
       <c r="AB96" s="14" t="inlineStr"/>
       <c r="AC96" s="15" t="n">
-        <v>0.68715</v>
+        <v>0.7827666666666667</v>
       </c>
       <c r="AD96" s="15" t="inlineStr"/>
       <c r="AE96" s="14" t="n">
-        <v>3.7542E7</v>
+        <v>2.6068E7</v>
       </c>
       <c r="AF96" s="14" t="inlineStr"/>
       <c r="AG96" s="14" t="inlineStr"/>
@@ -6370,23 +6370,23 @@
       <c r="U99" s="14" t="inlineStr"/>
       <c r="V99" s="14" t="inlineStr"/>
       <c r="W99" s="14" t="n">
-        <v>1.8974272E7</v>
+        <v>1.9186331E7</v>
       </c>
       <c r="X99" s="14" t="n">
-        <v>212059.0</v>
+        <v>198083.0</v>
       </c>
       <c r="Y99" s="14" t="inlineStr"/>
       <c r="Z99" s="14" t="n">
-        <v>1.9186331E7</v>
+        <v>1.9384414E7</v>
       </c>
       <c r="AA99" s="14" t="inlineStr"/>
       <c r="AB99" s="14" t="inlineStr"/>
       <c r="AC99" s="15" t="n">
-        <v>0.9690066161616162</v>
+        <v>0.9790108080808081</v>
       </c>
       <c r="AD99" s="15" t="inlineStr"/>
       <c r="AE99" s="14" t="n">
-        <v>613669.0</v>
+        <v>415586.0</v>
       </c>
       <c r="AF99" s="14" t="inlineStr"/>
       <c r="AG99" s="14" t="inlineStr"/>
@@ -6427,23 +6427,23 @@
       <c r="U100" s="14" t="inlineStr"/>
       <c r="V100" s="14" t="inlineStr"/>
       <c r="W100" s="14" t="n">
-        <v>1443256.0</v>
+        <v>1655315.0</v>
       </c>
       <c r="X100" s="14" t="n">
-        <v>212059.0</v>
+        <v>198083.0</v>
       </c>
       <c r="Y100" s="14" t="inlineStr"/>
       <c r="Z100" s="14" t="n">
-        <v>1655315.0</v>
+        <v>1853398.0</v>
       </c>
       <c r="AA100" s="14" t="inlineStr"/>
       <c r="AB100" s="14" t="inlineStr"/>
       <c r="AC100" s="15" t="n">
-        <v>0.6897145833333334</v>
+        <v>0.7722491666666667</v>
       </c>
       <c r="AD100" s="15" t="inlineStr"/>
       <c r="AE100" s="14" t="n">
-        <v>744685.0</v>
+        <v>546602.0</v>
       </c>
       <c r="AF100" s="14" t="inlineStr"/>
       <c r="AG100" s="14" t="inlineStr"/>
@@ -6604,23 +6604,23 @@
       <c r="U103" s="14" t="inlineStr"/>
       <c r="V103" s="14" t="inlineStr"/>
       <c r="W103" s="14" t="n">
-        <v>7.06095E7</v>
+        <v>7.864812E7</v>
       </c>
       <c r="X103" s="14" t="n">
-        <v>8038620.0</v>
+        <v>8617980.0</v>
       </c>
       <c r="Y103" s="14" t="inlineStr"/>
       <c r="Z103" s="14" t="n">
-        <v>7.864812E7</v>
+        <v>8.72661E7</v>
       </c>
       <c r="AA103" s="14" t="inlineStr"/>
       <c r="AB103" s="14" t="inlineStr"/>
       <c r="AC103" s="15" t="n">
-        <v>0.6241914285714286</v>
+        <v>0.6925880952380953</v>
       </c>
       <c r="AD103" s="15" t="inlineStr"/>
       <c r="AE103" s="14" t="n">
-        <v>4.735188E7</v>
+        <v>3.87339E7</v>
       </c>
       <c r="AF103" s="14" t="inlineStr"/>
       <c r="AG103" s="14" t="inlineStr"/>
@@ -6661,23 +6661,23 @@
       <c r="U104" s="14" t="inlineStr"/>
       <c r="V104" s="14" t="inlineStr"/>
       <c r="W104" s="14" t="n">
-        <v>5.308386E7</v>
+        <v>6.112248E7</v>
       </c>
       <c r="X104" s="14" t="n">
-        <v>8038620.0</v>
+        <v>8617980.0</v>
       </c>
       <c r="Y104" s="14" t="inlineStr"/>
       <c r="Z104" s="14" t="n">
-        <v>6.112248E7</v>
+        <v>6.974046E7</v>
       </c>
       <c r="AA104" s="14" t="inlineStr"/>
       <c r="AB104" s="14" t="inlineStr"/>
       <c r="AC104" s="15" t="n">
-        <v>0.5659488888888888</v>
+        <v>0.645745</v>
       </c>
       <c r="AD104" s="15" t="inlineStr"/>
       <c r="AE104" s="14" t="n">
-        <v>4.687752E7</v>
+        <v>3.825954E7</v>
       </c>
       <c r="AF104" s="14" t="inlineStr"/>
       <c r="AG104" s="14" t="inlineStr"/>
@@ -6838,10 +6838,10 @@
       <c r="U107" s="14" t="inlineStr"/>
       <c r="V107" s="14" t="inlineStr"/>
       <c r="W107" s="14" t="n">
-        <v>1.28383E8</v>
+        <v>1.54008E8</v>
       </c>
       <c r="X107" s="14" t="n">
-        <v>2.5625E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y107" s="14" t="inlineStr"/>
       <c r="Z107" s="14" t="n">
@@ -6895,10 +6895,10 @@
       <c r="U108" s="14" t="inlineStr"/>
       <c r="V108" s="14" t="inlineStr"/>
       <c r="W108" s="14" t="n">
-        <v>8260000.0</v>
+        <v>9450000.0</v>
       </c>
       <c r="X108" s="14" t="n">
-        <v>1190000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y108" s="14" t="inlineStr"/>
       <c r="Z108" s="14" t="n">
@@ -6952,10 +6952,10 @@
       <c r="U109" s="14" t="inlineStr"/>
       <c r="V109" s="14" t="inlineStr"/>
       <c r="W109" s="14" t="n">
-        <v>1.05117E8</v>
+        <v>1.25985E8</v>
       </c>
       <c r="X109" s="14" t="n">
-        <v>2.0868E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y109" s="14" t="inlineStr"/>
       <c r="Z109" s="14" t="n">
@@ -7009,10 +7009,10 @@
       <c r="U110" s="14" t="inlineStr"/>
       <c r="V110" s="14" t="inlineStr"/>
       <c r="W110" s="14" t="n">
-        <v>1.5006E7</v>
+        <v>1.8573E7</v>
       </c>
       <c r="X110" s="14" t="n">
-        <v>3567000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y110" s="14" t="inlineStr"/>
       <c r="Z110" s="14" t="n">
@@ -7072,23 +7072,23 @@
       <c r="U111" s="14" t="inlineStr"/>
       <c r="V111" s="14" t="inlineStr"/>
       <c r="W111" s="14" t="n">
-        <v>3.23E7</v>
+        <v>3.637E7</v>
       </c>
       <c r="X111" s="14" t="n">
         <v>4070000.0</v>
       </c>
       <c r="Y111" s="14" t="inlineStr"/>
       <c r="Z111" s="14" t="n">
-        <v>3.637E7</v>
+        <v>4.044E7</v>
       </c>
       <c r="AA111" s="14" t="inlineStr"/>
       <c r="AB111" s="14" t="inlineStr"/>
       <c r="AC111" s="15" t="n">
-        <v>0.5773015873015873</v>
+        <v>0.6419047619047619</v>
       </c>
       <c r="AD111" s="15" t="inlineStr"/>
       <c r="AE111" s="14" t="n">
-        <v>2.663E7</v>
+        <v>2.256E7</v>
       </c>
       <c r="AF111" s="14" t="inlineStr"/>
       <c r="AG111" s="14" t="inlineStr"/>
@@ -7129,23 +7129,23 @@
       <c r="U112" s="14" t="inlineStr"/>
       <c r="V112" s="14" t="inlineStr"/>
       <c r="W112" s="14" t="n">
-        <v>2.437E7</v>
+        <v>2.844E7</v>
       </c>
       <c r="X112" s="14" t="n">
         <v>4070000.0</v>
       </c>
       <c r="Y112" s="14" t="inlineStr"/>
       <c r="Z112" s="14" t="n">
-        <v>2.844E7</v>
+        <v>3.251E7</v>
       </c>
       <c r="AA112" s="14" t="inlineStr"/>
       <c r="AB112" s="14" t="inlineStr"/>
       <c r="AC112" s="15" t="n">
-        <v>0.5266666666666666</v>
+        <v>0.602037037037037</v>
       </c>
       <c r="AD112" s="15" t="inlineStr"/>
       <c r="AE112" s="14" t="n">
-        <v>2.556E7</v>
+        <v>2.149E7</v>
       </c>
       <c r="AF112" s="14" t="inlineStr"/>
       <c r="AG112" s="14" t="inlineStr"/>
@@ -7350,23 +7350,23 @@
       <c r="U116" s="14" t="inlineStr"/>
       <c r="V116" s="14" t="inlineStr"/>
       <c r="W116" s="14" t="n">
-        <v>1.569837989E9</v>
+        <v>1.753569219E9</v>
       </c>
       <c r="X116" s="14" t="n">
-        <v>1.8373123E8</v>
+        <v>1.82493718E8</v>
       </c>
       <c r="Y116" s="14" t="inlineStr"/>
       <c r="Z116" s="14" t="n">
-        <v>1.753569219E9</v>
+        <v>1.936062937E9</v>
       </c>
       <c r="AA116" s="14" t="inlineStr"/>
       <c r="AB116" s="14" t="inlineStr"/>
       <c r="AC116" s="15" t="n">
-        <v>0.6557850482423336</v>
+        <v>0.7240325119670905</v>
       </c>
       <c r="AD116" s="15" t="inlineStr"/>
       <c r="AE116" s="14" t="n">
-        <v>9.20430781E8</v>
+        <v>7.37937063E8</v>
       </c>
       <c r="AF116" s="14" t="inlineStr"/>
       <c r="AG116" s="14" t="inlineStr"/>
@@ -7407,23 +7407,23 @@
       <c r="U117" s="14" t="inlineStr"/>
       <c r="V117" s="14" t="inlineStr"/>
       <c r="W117" s="14" t="n">
-        <v>1.127223197E9</v>
+        <v>1.310954427E9</v>
       </c>
       <c r="X117" s="14" t="n">
-        <v>1.8373123E8</v>
+        <v>1.82493718E8</v>
       </c>
       <c r="Y117" s="14" t="inlineStr"/>
       <c r="Z117" s="14" t="n">
-        <v>1.310954427E9</v>
+        <v>1.493448145E9</v>
       </c>
       <c r="AA117" s="14" t="inlineStr"/>
       <c r="AB117" s="14" t="inlineStr"/>
       <c r="AC117" s="15" t="n">
-        <v>0.5879774071582347</v>
+        <v>0.6698278368317186</v>
       </c>
       <c r="AD117" s="15" t="inlineStr"/>
       <c r="AE117" s="14" t="n">
-        <v>9.18645573E8</v>
+        <v>7.36151855E8</v>
       </c>
       <c r="AF117" s="14" t="inlineStr"/>
       <c r="AG117" s="14" t="inlineStr"/>
@@ -9449,23 +9449,23 @@
       <c r="U152" s="14" t="inlineStr"/>
       <c r="V152" s="14" t="inlineStr"/>
       <c r="W152" s="14" t="n">
-        <v>2.9995561161E10</v>
+        <v>3.3898086196E10</v>
       </c>
       <c r="X152" s="14" t="n">
-        <v>3.902525035E9</v>
+        <v>1.646912991E9</v>
       </c>
       <c r="Y152" s="14" t="inlineStr"/>
       <c r="Z152" s="14" t="n">
-        <v>3.3898086196E10</v>
+        <v>3.5544999187E10</v>
       </c>
       <c r="AA152" s="14" t="inlineStr"/>
       <c r="AB152" s="14" t="inlineStr"/>
       <c r="AC152" s="15" t="n">
-        <v>0.640929169773647</v>
+        <v>0.672068230837679</v>
       </c>
       <c r="AD152" s="15" t="inlineStr"/>
       <c r="AE152" s="14" t="n">
-        <v>1.8990887804E10</v>
+        <v>1.7343974813E10</v>
       </c>
       <c r="AF152" s="14" t="inlineStr"/>
       <c r="AG152" s="14" t="inlineStr"/>
@@ -9512,23 +9512,23 @@
       <c r="U153" s="14" t="inlineStr"/>
       <c r="V153" s="14" t="inlineStr"/>
       <c r="W153" s="14" t="n">
-        <v>9.9508303E9</v>
+        <v>1.11880769E10</v>
       </c>
       <c r="X153" s="14" t="n">
-        <v>1.2372466E9</v>
+        <v>1.1951534E9</v>
       </c>
       <c r="Y153" s="14" t="inlineStr"/>
       <c r="Z153" s="14" t="n">
-        <v>1.11880769E10</v>
+        <v>1.23832303E10</v>
       </c>
       <c r="AA153" s="14" t="inlineStr"/>
       <c r="AB153" s="14" t="inlineStr"/>
       <c r="AC153" s="15" t="n">
-        <v>0.8507580690479567</v>
+        <v>0.9416393177101017</v>
       </c>
       <c r="AD153" s="15" t="inlineStr"/>
       <c r="AE153" s="14" t="n">
-        <v>1.9626381E9</v>
+        <v>7.674847E8</v>
       </c>
       <c r="AF153" s="14" t="inlineStr"/>
       <c r="AG153" s="14" t="inlineStr"/>
@@ -9569,23 +9569,23 @@
       <c r="U154" s="14" t="inlineStr"/>
       <c r="V154" s="14" t="inlineStr"/>
       <c r="W154" s="14" t="n">
-        <v>7.4634674E9</v>
+        <v>8.6973235E9</v>
       </c>
       <c r="X154" s="14" t="n">
-        <v>1.2338561E9</v>
+        <v>1.1951534E9</v>
       </c>
       <c r="Y154" s="14" t="inlineStr"/>
       <c r="Z154" s="14" t="n">
-        <v>8.6973235E9</v>
+        <v>9.8924769E9</v>
       </c>
       <c r="AA154" s="14" t="inlineStr"/>
       <c r="AB154" s="14" t="inlineStr"/>
       <c r="AC154" s="15" t="n">
-        <v>0.8207115758585963</v>
+        <v>0.933490665920816</v>
       </c>
       <c r="AD154" s="15" t="inlineStr"/>
       <c r="AE154" s="14" t="n">
-        <v>1.8999725E9</v>
+        <v>7.048191E8</v>
       </c>
       <c r="AF154" s="14" t="inlineStr"/>
       <c r="AG154" s="14" t="inlineStr"/>
@@ -9626,10 +9626,10 @@
       <c r="U155" s="14" t="inlineStr"/>
       <c r="V155" s="14" t="inlineStr"/>
       <c r="W155" s="14" t="n">
-        <v>1.2339441E9</v>
+        <v>1.2373346E9</v>
       </c>
       <c r="X155" s="14" t="n">
-        <v>3390500.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y155" s="14" t="inlineStr"/>
       <c r="Z155" s="14" t="n">
@@ -9746,23 +9746,23 @@
       <c r="U157" s="14" t="inlineStr"/>
       <c r="V157" s="14" t="inlineStr"/>
       <c r="W157" s="14" t="n">
-        <v>135783.0</v>
+        <v>152199.0</v>
       </c>
       <c r="X157" s="14" t="n">
-        <v>16416.0</v>
+        <v>15915.0</v>
       </c>
       <c r="Y157" s="14" t="inlineStr"/>
       <c r="Z157" s="14" t="n">
-        <v>152199.0</v>
+        <v>168114.0</v>
       </c>
       <c r="AA157" s="14" t="inlineStr"/>
       <c r="AB157" s="14" t="inlineStr"/>
       <c r="AC157" s="15" t="n">
-        <v>0.6394915966386555</v>
+        <v>0.7063613445378151</v>
       </c>
       <c r="AD157" s="15" t="inlineStr"/>
       <c r="AE157" s="14" t="n">
-        <v>85801.0</v>
+        <v>69886.0</v>
       </c>
       <c r="AF157" s="14" t="inlineStr"/>
       <c r="AG157" s="14" t="inlineStr"/>
@@ -9803,23 +9803,23 @@
       <c r="U158" s="14" t="inlineStr"/>
       <c r="V158" s="14" t="inlineStr"/>
       <c r="W158" s="14" t="n">
-        <v>102089.0</v>
+        <v>118425.0</v>
       </c>
       <c r="X158" s="14" t="n">
-        <v>16336.0</v>
+        <v>15915.0</v>
       </c>
       <c r="Y158" s="14" t="inlineStr"/>
       <c r="Z158" s="14" t="n">
-        <v>118425.0</v>
+        <v>134340.0</v>
       </c>
       <c r="AA158" s="14" t="inlineStr"/>
       <c r="AB158" s="14" t="inlineStr"/>
       <c r="AC158" s="15" t="n">
-        <v>0.580514705882353</v>
+        <v>0.6585294117647059</v>
       </c>
       <c r="AD158" s="15" t="inlineStr"/>
       <c r="AE158" s="14" t="n">
-        <v>85575.0</v>
+        <v>69660.0</v>
       </c>
       <c r="AF158" s="14" t="inlineStr"/>
       <c r="AG158" s="14" t="inlineStr"/>
@@ -9860,10 +9860,10 @@
       <c r="U159" s="14" t="inlineStr"/>
       <c r="V159" s="14" t="inlineStr"/>
       <c r="W159" s="14" t="n">
-        <v>16986.0</v>
+        <v>17066.0</v>
       </c>
       <c r="X159" s="14" t="n">
-        <v>80.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y159" s="14" t="inlineStr"/>
       <c r="Z159" s="14" t="n">
@@ -9980,23 +9980,23 @@
       <c r="U161" s="14" t="inlineStr"/>
       <c r="V161" s="14" t="inlineStr"/>
       <c r="W161" s="14" t="n">
-        <v>7.8074705E8</v>
+        <v>8.786895E8</v>
       </c>
       <c r="X161" s="14" t="n">
-        <v>9.794245E7</v>
+        <v>9.460116E7</v>
       </c>
       <c r="Y161" s="14" t="inlineStr"/>
       <c r="Z161" s="14" t="n">
-        <v>8.786895E8</v>
+        <v>9.7329066E8</v>
       </c>
       <c r="AA161" s="14" t="inlineStr"/>
       <c r="AB161" s="14" t="inlineStr"/>
       <c r="AC161" s="15" t="n">
-        <v>0.6406543691443987</v>
+        <v>0.7096282745798549</v>
       </c>
       <c r="AD161" s="15" t="inlineStr"/>
       <c r="AE161" s="14" t="n">
-        <v>4.928605E8</v>
+        <v>3.9825934E8</v>
       </c>
       <c r="AF161" s="14" t="inlineStr"/>
       <c r="AG161" s="14" t="inlineStr"/>
@@ -10037,23 +10037,23 @@
       <c r="U162" s="14" t="inlineStr"/>
       <c r="V162" s="14" t="inlineStr"/>
       <c r="W162" s="14" t="n">
-        <v>5.8576199E8</v>
+        <v>6.8370444E8</v>
       </c>
       <c r="X162" s="14" t="n">
-        <v>9.794245E7</v>
+        <v>9.460116E7</v>
       </c>
       <c r="Y162" s="14" t="inlineStr"/>
       <c r="Z162" s="14" t="n">
-        <v>6.8370444E8</v>
+        <v>7.783056E8</v>
       </c>
       <c r="AA162" s="14" t="inlineStr"/>
       <c r="AB162" s="14" t="inlineStr"/>
       <c r="AC162" s="15" t="n">
-        <v>0.5813813265306123</v>
+        <v>0.6618244897959183</v>
       </c>
       <c r="AD162" s="15" t="inlineStr"/>
       <c r="AE162" s="14" t="n">
-        <v>4.9229556E8</v>
+        <v>3.976944E8</v>
       </c>
       <c r="AF162" s="14" t="inlineStr"/>
       <c r="AG162" s="14" t="inlineStr"/>
@@ -10214,23 +10214,23 @@
       <c r="U165" s="14" t="inlineStr"/>
       <c r="V165" s="14" t="inlineStr"/>
       <c r="W165" s="14" t="n">
-        <v>2.4201339E8</v>
+        <v>2.7256082E8</v>
       </c>
       <c r="X165" s="14" t="n">
-        <v>3.054743E7</v>
+        <v>2.9746002E7</v>
       </c>
       <c r="Y165" s="14" t="inlineStr"/>
       <c r="Z165" s="14" t="n">
-        <v>2.7256082E8</v>
+        <v>3.02306822E8</v>
       </c>
       <c r="AA165" s="14" t="inlineStr"/>
       <c r="AB165" s="14" t="inlineStr"/>
       <c r="AC165" s="15" t="n">
-        <v>0.6290973256058182</v>
+        <v>0.6977540397500791</v>
       </c>
       <c r="AD165" s="15" t="inlineStr"/>
       <c r="AE165" s="14" t="n">
-        <v>1.6069618E8</v>
+        <v>1.30950178E8</v>
       </c>
       <c r="AF165" s="14" t="inlineStr"/>
       <c r="AG165" s="14" t="inlineStr"/>
@@ -10271,23 +10271,23 @@
       <c r="U166" s="14" t="inlineStr"/>
       <c r="V166" s="14" t="inlineStr"/>
       <c r="W166" s="14" t="n">
-        <v>1.81690344E8</v>
+        <v>2.12169964E8</v>
       </c>
       <c r="X166" s="14" t="n">
-        <v>3.047962E7</v>
+        <v>2.9746002E7</v>
       </c>
       <c r="Y166" s="14" t="inlineStr"/>
       <c r="Z166" s="14" t="n">
-        <v>2.12169964E8</v>
+        <v>2.41915966E8</v>
       </c>
       <c r="AA166" s="14" t="inlineStr"/>
       <c r="AB166" s="14" t="inlineStr"/>
       <c r="AC166" s="15" t="n">
-        <v>0.5703493655913978</v>
+        <v>0.6503117365591398</v>
       </c>
       <c r="AD166" s="15" t="inlineStr"/>
       <c r="AE166" s="14" t="n">
-        <v>1.59830036E8</v>
+        <v>1.30084034E8</v>
       </c>
       <c r="AF166" s="14" t="inlineStr"/>
       <c r="AG166" s="14" t="inlineStr"/>
@@ -10328,10 +10328,10 @@
       <c r="U167" s="14" t="inlineStr"/>
       <c r="V167" s="14" t="inlineStr"/>
       <c r="W167" s="14" t="n">
-        <v>3.0066354E7</v>
+        <v>3.0134164E7</v>
       </c>
       <c r="X167" s="14" t="n">
-        <v>67810.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y167" s="14" t="inlineStr"/>
       <c r="Z167" s="14" t="n">
@@ -10492,23 +10492,23 @@
       <c r="U170" s="14" t="inlineStr"/>
       <c r="V170" s="14" t="inlineStr"/>
       <c r="W170" s="14" t="n">
-        <v>2.15166E9</v>
+        <v>2.41703E9</v>
       </c>
       <c r="X170" s="14" t="n">
-        <v>2.6537E8</v>
+        <v>2.5728E8</v>
       </c>
       <c r="Y170" s="14" t="inlineStr"/>
       <c r="Z170" s="14" t="n">
-        <v>2.41703E9</v>
+        <v>2.67431E9</v>
       </c>
       <c r="AA170" s="14" t="inlineStr"/>
       <c r="AB170" s="14" t="inlineStr"/>
       <c r="AC170" s="15" t="n">
-        <v>0.6278</v>
+        <v>0.694625974025974</v>
       </c>
       <c r="AD170" s="15" t="inlineStr"/>
       <c r="AE170" s="14" t="n">
-        <v>1.43297E9</v>
+        <v>1.17569E9</v>
       </c>
       <c r="AF170" s="14" t="inlineStr"/>
       <c r="AG170" s="14" t="inlineStr"/>
@@ -10549,23 +10549,23 @@
       <c r="U171" s="14" t="inlineStr"/>
       <c r="V171" s="14" t="inlineStr"/>
       <c r="W171" s="14" t="n">
-        <v>1.61394E9</v>
+        <v>1.87877E9</v>
       </c>
       <c r="X171" s="14" t="n">
-        <v>2.6483E8</v>
+        <v>2.5728E8</v>
       </c>
       <c r="Y171" s="14" t="inlineStr"/>
       <c r="Z171" s="14" t="n">
-        <v>1.87877E9</v>
+        <v>2.13605E9</v>
       </c>
       <c r="AA171" s="14" t="inlineStr"/>
       <c r="AB171" s="14" t="inlineStr"/>
       <c r="AC171" s="15" t="n">
-        <v>0.5693242424242424</v>
+        <v>0.6472878787878787</v>
       </c>
       <c r="AD171" s="15" t="inlineStr"/>
       <c r="AE171" s="14" t="n">
-        <v>1.42123E9</v>
+        <v>1.16395E9</v>
       </c>
       <c r="AF171" s="14" t="inlineStr"/>
       <c r="AG171" s="14" t="inlineStr"/>
@@ -10606,10 +10606,10 @@
       <c r="U172" s="14" t="inlineStr"/>
       <c r="V172" s="14" t="inlineStr"/>
       <c r="W172" s="14" t="n">
-        <v>2.6553E8</v>
+        <v>2.6607E8</v>
       </c>
       <c r="X172" s="14" t="n">
-        <v>540000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y172" s="14" t="inlineStr"/>
       <c r="Z172" s="14" t="n">
@@ -10726,23 +10726,23 @@
       <c r="U174" s="14" t="inlineStr"/>
       <c r="V174" s="14" t="inlineStr"/>
       <c r="W174" s="14" t="n">
-        <v>2.10388789E8</v>
+        <v>2.14257962E8</v>
       </c>
       <c r="X174" s="14" t="n">
-        <v>3869173.0</v>
+        <v>3377534.0</v>
       </c>
       <c r="Y174" s="14" t="inlineStr"/>
       <c r="Z174" s="14" t="n">
-        <v>2.14257962E8</v>
+        <v>2.17635496E8</v>
       </c>
       <c r="AA174" s="14" t="inlineStr"/>
       <c r="AB174" s="14" t="inlineStr"/>
       <c r="AC174" s="15" t="n">
-        <v>0.8719243153054165</v>
+        <v>0.885669214178163</v>
       </c>
       <c r="AD174" s="15" t="inlineStr"/>
       <c r="AE174" s="14" t="n">
-        <v>3.1472038E7</v>
+        <v>2.8094504E7</v>
       </c>
       <c r="AF174" s="14" t="inlineStr"/>
       <c r="AG174" s="14" t="inlineStr"/>
@@ -10783,23 +10783,23 @@
       <c r="U175" s="14" t="inlineStr"/>
       <c r="V175" s="14" t="inlineStr"/>
       <c r="W175" s="14" t="n">
-        <v>2.5023751E7</v>
+        <v>2.8801831E7</v>
       </c>
       <c r="X175" s="14" t="n">
-        <v>3778080.0</v>
+        <v>3377534.0</v>
       </c>
       <c r="Y175" s="14" t="inlineStr"/>
       <c r="Z175" s="14" t="n">
-        <v>2.8801831E7</v>
+        <v>3.2179365E7</v>
       </c>
       <c r="AA175" s="14" t="inlineStr"/>
       <c r="AB175" s="14" t="inlineStr"/>
       <c r="AC175" s="15" t="n">
-        <v>0.4800305166666667</v>
+        <v>0.53632275</v>
       </c>
       <c r="AD175" s="15" t="inlineStr"/>
       <c r="AE175" s="14" t="n">
-        <v>3.1198169E7</v>
+        <v>2.7820635E7</v>
       </c>
       <c r="AF175" s="14" t="inlineStr"/>
       <c r="AG175" s="14" t="inlineStr"/>
@@ -10840,10 +10840,10 @@
       <c r="U176" s="14" t="inlineStr"/>
       <c r="V176" s="14" t="inlineStr"/>
       <c r="W176" s="14" t="n">
-        <v>9.2637075E7</v>
+        <v>9.2728168E7</v>
       </c>
       <c r="X176" s="14" t="n">
-        <v>91093.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y176" s="14" t="inlineStr"/>
       <c r="Z176" s="14" t="n">
@@ -10960,23 +10960,23 @@
       <c r="U178" s="14" t="inlineStr"/>
       <c r="V178" s="14" t="inlineStr"/>
       <c r="W178" s="14" t="n">
-        <v>5.449605E8</v>
+        <v>6.133974E8</v>
       </c>
       <c r="X178" s="14" t="n">
-        <v>6.84369E7</v>
+        <v>6.655398E7</v>
       </c>
       <c r="Y178" s="14" t="inlineStr"/>
       <c r="Z178" s="14" t="n">
-        <v>6.133974E8</v>
+        <v>6.7995138E8</v>
       </c>
       <c r="AA178" s="14" t="inlineStr"/>
       <c r="AB178" s="14" t="inlineStr"/>
       <c r="AC178" s="15" t="n">
-        <v>0.6259157142857142</v>
+        <v>0.6938279387755102</v>
       </c>
       <c r="AD178" s="15" t="inlineStr"/>
       <c r="AE178" s="14" t="n">
-        <v>3.666026E8</v>
+        <v>3.0004862E8</v>
       </c>
       <c r="AF178" s="14" t="inlineStr"/>
       <c r="AG178" s="14" t="inlineStr"/>
@@ -11017,23 +11017,23 @@
       <c r="U179" s="14" t="inlineStr"/>
       <c r="V179" s="14" t="inlineStr"/>
       <c r="W179" s="14" t="n">
-        <v>4.084488E8</v>
+        <v>4.7666844E8</v>
       </c>
       <c r="X179" s="14" t="n">
-        <v>6.821964E7</v>
+        <v>6.655398E7</v>
       </c>
       <c r="Y179" s="14" t="inlineStr"/>
       <c r="Z179" s="14" t="n">
-        <v>4.7666844E8</v>
+        <v>5.4322242E8</v>
       </c>
       <c r="AA179" s="14" t="inlineStr"/>
       <c r="AB179" s="14" t="inlineStr"/>
       <c r="AC179" s="15" t="n">
-        <v>0.5674624285714286</v>
+        <v>0.6466933571428571</v>
       </c>
       <c r="AD179" s="15" t="inlineStr"/>
       <c r="AE179" s="14" t="n">
-        <v>3.6333156E8</v>
+        <v>2.9677758E8</v>
       </c>
       <c r="AF179" s="14" t="inlineStr"/>
       <c r="AG179" s="14" t="inlineStr"/>
@@ -11074,10 +11074,10 @@
       <c r="U180" s="14" t="inlineStr"/>
       <c r="V180" s="14" t="inlineStr"/>
       <c r="W180" s="14" t="n">
-        <v>6.778512E7</v>
+        <v>6.800238E7</v>
       </c>
       <c r="X180" s="14" t="n">
-        <v>217260.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y180" s="14" t="inlineStr"/>
       <c r="Z180" s="14" t="n">
@@ -11194,10 +11194,10 @@
       <c r="U182" s="14" t="inlineStr"/>
       <c r="V182" s="14" t="inlineStr"/>
       <c r="W182" s="14" t="n">
-        <v>1.046634E9</v>
+        <v>1.249247E9</v>
       </c>
       <c r="X182" s="14" t="n">
-        <v>2.02613E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y182" s="14" t="inlineStr"/>
       <c r="Z182" s="14" t="n">
@@ -11251,10 +11251,10 @@
       <c r="U183" s="14" t="inlineStr"/>
       <c r="V183" s="14" t="inlineStr"/>
       <c r="W183" s="14" t="n">
-        <v>9.1E7</v>
+        <v>1.09165E8</v>
       </c>
       <c r="X183" s="14" t="n">
-        <v>1.8165E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y183" s="14" t="inlineStr"/>
       <c r="Z183" s="14" t="n">
@@ -11308,10 +11308,10 @@
       <c r="U184" s="14" t="inlineStr"/>
       <c r="V184" s="14" t="inlineStr"/>
       <c r="W184" s="14" t="n">
-        <v>7.40999E8</v>
+        <v>8.87112E8</v>
       </c>
       <c r="X184" s="14" t="n">
-        <v>1.46113E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y184" s="14" t="inlineStr"/>
       <c r="Z184" s="14" t="n">
@@ -11365,10 +11365,10 @@
       <c r="U185" s="14" t="inlineStr"/>
       <c r="V185" s="14" t="inlineStr"/>
       <c r="W185" s="14" t="n">
-        <v>2.14635E8</v>
+        <v>2.5297E8</v>
       </c>
       <c r="X185" s="14" t="n">
-        <v>3.8335E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y185" s="14" t="inlineStr"/>
       <c r="Z185" s="14" t="n">
@@ -11428,23 +11428,23 @@
       <c r="U186" s="14" t="inlineStr"/>
       <c r="V186" s="14" t="inlineStr"/>
       <c r="W186" s="14" t="n">
-        <v>1850000.0</v>
+        <v>2035000.0</v>
       </c>
       <c r="X186" s="14" t="n">
         <v>185000.0</v>
       </c>
       <c r="Y186" s="14" t="inlineStr"/>
       <c r="Z186" s="14" t="n">
-        <v>2035000.0</v>
+        <v>2220000.0</v>
       </c>
       <c r="AA186" s="14" t="inlineStr"/>
       <c r="AB186" s="14" t="inlineStr"/>
       <c r="AC186" s="15" t="n">
-        <v>0.39285714285714285</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="AD186" s="15" t="inlineStr"/>
       <c r="AE186" s="14" t="n">
-        <v>3145000.0</v>
+        <v>2960000.0</v>
       </c>
       <c r="AF186" s="14" t="inlineStr"/>
       <c r="AG186" s="14" t="inlineStr"/>
@@ -11485,23 +11485,23 @@
       <c r="U187" s="14" t="inlineStr"/>
       <c r="V187" s="14" t="inlineStr"/>
       <c r="W187" s="14" t="n">
-        <v>1295000.0</v>
+        <v>1480000.0</v>
       </c>
       <c r="X187" s="14" t="n">
         <v>185000.0</v>
       </c>
       <c r="Y187" s="14" t="inlineStr"/>
       <c r="Z187" s="14" t="n">
-        <v>1480000.0</v>
+        <v>1665000.0</v>
       </c>
       <c r="AA187" s="14" t="inlineStr"/>
       <c r="AB187" s="14" t="inlineStr"/>
       <c r="AC187" s="15" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.375</v>
       </c>
       <c r="AD187" s="15" t="inlineStr"/>
       <c r="AE187" s="14" t="n">
-        <v>2960000.0</v>
+        <v>2775000.0</v>
       </c>
       <c r="AF187" s="14" t="inlineStr"/>
       <c r="AG187" s="14" t="inlineStr"/>
@@ -11662,10 +11662,10 @@
       <c r="U190" s="14" t="inlineStr"/>
       <c r="V190" s="14" t="inlineStr"/>
       <c r="W190" s="14" t="n">
-        <v>1.5066341349E10</v>
+        <v>1.7062639415E10</v>
       </c>
       <c r="X190" s="14" t="n">
-        <v>1.996298066E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y190" s="14" t="inlineStr"/>
       <c r="Z190" s="14" t="n">
@@ -11719,10 +11719,10 @@
       <c r="U191" s="14" t="inlineStr"/>
       <c r="V191" s="14" t="inlineStr"/>
       <c r="W191" s="14" t="n">
-        <v>1.0293742797E10</v>
+        <v>1.2285354215E10</v>
       </c>
       <c r="X191" s="14" t="n">
-        <v>1.991611418E9</v>
+        <v>0.0</v>
       </c>
       <c r="Y191" s="14" t="inlineStr"/>
       <c r="Z191" s="14" t="n">
@@ -11776,10 +11776,10 @@
       <c r="U192" s="14" t="inlineStr"/>
       <c r="V192" s="14" t="inlineStr"/>
       <c r="W192" s="14" t="n">
-        <v>2.362459773E9</v>
+        <v>2.367146421E9</v>
       </c>
       <c r="X192" s="14" t="n">
-        <v>4686648.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y192" s="14" t="inlineStr"/>
       <c r="Z192" s="14" t="n">
@@ -11896,23 +11896,23 @@
       <c r="U194" s="14" t="inlineStr"/>
       <c r="V194" s="14" t="inlineStr"/>
       <c r="W194" s="14" t="n">
-        <v>1.1289104178E10</v>
+        <v>1.2877655972E10</v>
       </c>
       <c r="X194" s="14" t="n">
-        <v>1.588551794E9</v>
+        <v>7.19581582E8</v>
       </c>
       <c r="Y194" s="14" t="inlineStr"/>
       <c r="Z194" s="14" t="n">
-        <v>1.2877655972E10</v>
+        <v>1.3597237554E10</v>
       </c>
       <c r="AA194" s="14" t="inlineStr"/>
       <c r="AB194" s="14" t="inlineStr"/>
       <c r="AC194" s="15" t="n">
-        <v>0.8588546270678621</v>
+        <v>0.9068459674637595</v>
       </c>
       <c r="AD194" s="15" t="inlineStr"/>
       <c r="AE194" s="14" t="n">
-        <v>2.116332028E9</v>
+        <v>1.396750446E9</v>
       </c>
       <c r="AF194" s="14" t="inlineStr"/>
       <c r="AG194" s="14" t="inlineStr"/>
@@ -12003,23 +12003,23 @@
       <c r="U196" s="14" t="inlineStr"/>
       <c r="V196" s="14" t="inlineStr"/>
       <c r="W196" s="14" t="n">
-        <v>4.219166866E9</v>
+        <v>4.762388866E9</v>
       </c>
       <c r="X196" s="14" t="n">
-        <v>5.43222E8</v>
+        <v>5.493708E8</v>
       </c>
       <c r="Y196" s="14" t="inlineStr"/>
       <c r="Z196" s="14" t="n">
-        <v>4.762388866E9</v>
+        <v>5.311759666E9</v>
       </c>
       <c r="AA196" s="14" t="inlineStr"/>
       <c r="AB196" s="14" t="inlineStr"/>
       <c r="AC196" s="15" t="n">
-        <v>1.0681407538457328</v>
+        <v>1.1913573489125906</v>
       </c>
       <c r="AD196" s="15" t="inlineStr"/>
       <c r="AE196" s="14" t="n">
-        <v>-3.03810866E8</v>
+        <v>-8.53181666E8</v>
       </c>
       <c r="AF196" s="14" t="inlineStr"/>
       <c r="AG196" s="14" t="inlineStr"/>
@@ -12060,23 +12060,23 @@
       <c r="U197" s="14" t="inlineStr"/>
       <c r="V197" s="14" t="inlineStr"/>
       <c r="W197" s="14" t="n">
-        <v>3.1300532E9</v>
+        <v>3.6732752E9</v>
       </c>
       <c r="X197" s="14" t="n">
-        <v>5.43222E8</v>
+        <v>5.493708E8</v>
       </c>
       <c r="Y197" s="14" t="inlineStr"/>
       <c r="Z197" s="14" t="n">
-        <v>3.6732752E9</v>
+        <v>4.222646E9</v>
       </c>
       <c r="AA197" s="14" t="inlineStr"/>
       <c r="AB197" s="14" t="inlineStr"/>
       <c r="AC197" s="15" t="n">
-        <v>1.091031224976179</v>
+        <v>1.2542045959477153</v>
       </c>
       <c r="AD197" s="15" t="inlineStr"/>
       <c r="AE197" s="14" t="n">
-        <v>-3.064832E8</v>
+        <v>-8.55854E8</v>
       </c>
       <c r="AF197" s="14" t="inlineStr"/>
       <c r="AG197" s="14" t="inlineStr"/>
@@ -12237,23 +12237,23 @@
       <c r="U200" s="14" t="inlineStr"/>
       <c r="V200" s="14" t="inlineStr"/>
       <c r="W200" s="14" t="n">
-        <v>80109.0</v>
+        <v>91671.0</v>
       </c>
       <c r="X200" s="14" t="n">
-        <v>11562.0</v>
+        <v>10062.0</v>
       </c>
       <c r="Y200" s="14" t="inlineStr"/>
       <c r="Z200" s="14" t="n">
-        <v>91671.0</v>
+        <v>101733.0</v>
       </c>
       <c r="AA200" s="14" t="inlineStr"/>
       <c r="AB200" s="14" t="inlineStr"/>
       <c r="AC200" s="15" t="n">
-        <v>0.5801962025316456</v>
+        <v>0.643879746835443</v>
       </c>
       <c r="AD200" s="15" t="inlineStr"/>
       <c r="AE200" s="14" t="n">
-        <v>66329.0</v>
+        <v>56267.0</v>
       </c>
       <c r="AF200" s="14" t="inlineStr"/>
       <c r="AG200" s="14" t="inlineStr"/>
@@ -12294,23 +12294,23 @@
       <c r="U201" s="14" t="inlineStr"/>
       <c r="V201" s="14" t="inlineStr"/>
       <c r="W201" s="14" t="n">
-        <v>66989.0</v>
+        <v>78551.0</v>
       </c>
       <c r="X201" s="14" t="n">
-        <v>11562.0</v>
+        <v>10062.0</v>
       </c>
       <c r="Y201" s="14" t="inlineStr"/>
       <c r="Z201" s="14" t="n">
-        <v>78551.0</v>
+        <v>88613.0</v>
       </c>
       <c r="AA201" s="14" t="inlineStr"/>
       <c r="AB201" s="14" t="inlineStr"/>
       <c r="AC201" s="15" t="n">
-        <v>0.5454930555555556</v>
+        <v>0.6153680555555555</v>
       </c>
       <c r="AD201" s="15" t="inlineStr"/>
       <c r="AE201" s="14" t="n">
-        <v>65449.0</v>
+        <v>55387.0</v>
       </c>
       <c r="AF201" s="14" t="inlineStr"/>
       <c r="AG201" s="14" t="inlineStr"/>
@@ -12471,23 +12471,23 @@
       <c r="U204" s="14" t="inlineStr"/>
       <c r="V204" s="14" t="inlineStr"/>
       <c r="W204" s="14" t="n">
-        <v>2.8535144E8</v>
+        <v>3.2254353E8</v>
       </c>
       <c r="X204" s="14" t="n">
-        <v>3.719209E7</v>
+        <v>3.730664E7</v>
       </c>
       <c r="Y204" s="14" t="inlineStr"/>
       <c r="Z204" s="14" t="n">
-        <v>3.2254353E8</v>
+        <v>3.5985017E8</v>
       </c>
       <c r="AA204" s="14" t="inlineStr"/>
       <c r="AB204" s="14" t="inlineStr"/>
       <c r="AC204" s="15" t="n">
-        <v>0.8933090626090521</v>
+        <v>0.9966326654960589</v>
       </c>
       <c r="AD204" s="15" t="inlineStr"/>
       <c r="AE204" s="14" t="n">
-        <v>3.852247E7</v>
+        <v>1215830.0</v>
       </c>
       <c r="AF204" s="14" t="inlineStr"/>
       <c r="AG204" s="14" t="inlineStr"/>
@@ -12528,23 +12528,23 @@
       <c r="U205" s="14" t="inlineStr"/>
       <c r="V205" s="14" t="inlineStr"/>
       <c r="W205" s="14" t="n">
-        <v>2.1196572E8</v>
+        <v>2.4881876E8</v>
       </c>
       <c r="X205" s="14" t="n">
-        <v>3.685304E7</v>
+        <v>3.730664E7</v>
       </c>
       <c r="Y205" s="14" t="inlineStr"/>
       <c r="Z205" s="14" t="n">
-        <v>2.4881876E8</v>
+        <v>2.861254E8</v>
       </c>
       <c r="AA205" s="14" t="inlineStr"/>
       <c r="AB205" s="14" t="inlineStr"/>
       <c r="AC205" s="15" t="n">
-        <v>0.8639540277777777</v>
+        <v>0.9934909722222223</v>
       </c>
       <c r="AD205" s="15" t="inlineStr"/>
       <c r="AE205" s="14" t="n">
-        <v>3.918124E7</v>
+        <v>1874600.0</v>
       </c>
       <c r="AF205" s="14" t="inlineStr"/>
       <c r="AG205" s="14" t="inlineStr"/>
@@ -12585,10 +12585,10 @@
       <c r="U206" s="14" t="inlineStr"/>
       <c r="V206" s="14" t="inlineStr"/>
       <c r="W206" s="14" t="n">
-        <v>3.685304E7</v>
+        <v>3.719209E7</v>
       </c>
       <c r="X206" s="14" t="n">
-        <v>339050.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y206" s="14" t="inlineStr"/>
       <c r="Z206" s="14" t="n">
@@ -12705,23 +12705,23 @@
       <c r="U208" s="14" t="inlineStr"/>
       <c r="V208" s="14" t="inlineStr"/>
       <c r="W208" s="14" t="n">
-        <v>8.5898944E7</v>
+        <v>9.6747576E7</v>
       </c>
       <c r="X208" s="14" t="n">
-        <v>1.0848632E7</v>
+        <v>1.098572E7</v>
       </c>
       <c r="Y208" s="14" t="inlineStr"/>
       <c r="Z208" s="14" t="n">
-        <v>9.6747576E7</v>
+        <v>1.07733296E8</v>
       </c>
       <c r="AA208" s="14" t="inlineStr"/>
       <c r="AB208" s="14" t="inlineStr"/>
       <c r="AC208" s="15" t="n">
-        <v>0.8632935003747725</v>
+        <v>0.9613207695327837</v>
       </c>
       <c r="AD208" s="15" t="inlineStr"/>
       <c r="AE208" s="14" t="n">
-        <v>1.5320424E7</v>
+        <v>4334704.0</v>
       </c>
       <c r="AF208" s="14" t="inlineStr"/>
       <c r="AG208" s="14" t="inlineStr"/>
@@ -12762,23 +12762,23 @@
       <c r="U209" s="14" t="inlineStr"/>
       <c r="V209" s="14" t="inlineStr"/>
       <c r="W209" s="14" t="n">
-        <v>6.401636E7</v>
+        <v>7.4864992E7</v>
       </c>
       <c r="X209" s="14" t="n">
-        <v>1.0848632E7</v>
+        <v>1.098572E7</v>
       </c>
       <c r="Y209" s="14" t="inlineStr"/>
       <c r="Z209" s="14" t="n">
-        <v>7.4864992E7</v>
+        <v>8.5850712E7</v>
       </c>
       <c r="AA209" s="14" t="inlineStr"/>
       <c r="AB209" s="14" t="inlineStr"/>
       <c r="AC209" s="15" t="n">
-        <v>0.8318332444444444</v>
+        <v>0.9538968</v>
       </c>
       <c r="AD209" s="15" t="inlineStr"/>
       <c r="AE209" s="14" t="n">
-        <v>1.5135008E7</v>
+        <v>4149288.0</v>
       </c>
       <c r="AF209" s="14" t="inlineStr"/>
       <c r="AG209" s="14" t="inlineStr"/>
@@ -12939,23 +12939,23 @@
       <c r="U212" s="14" t="inlineStr"/>
       <c r="V212" s="14" t="inlineStr"/>
       <c r="W212" s="14" t="n">
-        <v>6.8943E8</v>
+        <v>7.7817E8</v>
       </c>
       <c r="X212" s="14" t="n">
         <v>8.874E7</v>
       </c>
       <c r="Y212" s="14" t="inlineStr"/>
       <c r="Z212" s="14" t="n">
-        <v>7.7817E8</v>
+        <v>8.6691E8</v>
       </c>
       <c r="AA212" s="14" t="inlineStr"/>
       <c r="AB212" s="14" t="inlineStr"/>
       <c r="AC212" s="15" t="n">
-        <v>0.8664239428151513</v>
+        <v>0.9652281381521812</v>
       </c>
       <c r="AD212" s="15" t="inlineStr"/>
       <c r="AE212" s="14" t="n">
-        <v>1.1997E8</v>
+        <v>3.123E7</v>
       </c>
       <c r="AF212" s="14" t="inlineStr"/>
       <c r="AG212" s="14" t="inlineStr"/>
@@ -12996,23 +12996,23 @@
       <c r="U213" s="14" t="inlineStr"/>
       <c r="V213" s="14" t="inlineStr"/>
       <c r="W213" s="14" t="n">
-        <v>5.1162E8</v>
+        <v>6.0036E8</v>
       </c>
       <c r="X213" s="14" t="n">
         <v>8.874E7</v>
       </c>
       <c r="Y213" s="14" t="inlineStr"/>
       <c r="Z213" s="14" t="n">
-        <v>6.0036E8</v>
+        <v>6.891E8</v>
       </c>
       <c r="AA213" s="14" t="inlineStr"/>
       <c r="AB213" s="14" t="inlineStr"/>
       <c r="AC213" s="15" t="n">
-        <v>0.8338333333333333</v>
+        <v>0.9570833333333333</v>
       </c>
       <c r="AD213" s="15" t="inlineStr"/>
       <c r="AE213" s="14" t="n">
-        <v>1.1964E8</v>
+        <v>3.09E7</v>
       </c>
       <c r="AF213" s="14" t="inlineStr"/>
       <c r="AG213" s="14" t="inlineStr"/>
@@ -13173,23 +13173,23 @@
       <c r="U216" s="14" t="inlineStr"/>
       <c r="V216" s="14" t="inlineStr"/>
       <c r="W216" s="14" t="n">
-        <v>2.5925153E8</v>
+        <v>2.9241989E8</v>
       </c>
       <c r="X216" s="14" t="n">
         <v>3.316836E7</v>
       </c>
       <c r="Y216" s="14" t="inlineStr"/>
       <c r="Z216" s="14" t="n">
-        <v>2.9241989E8</v>
+        <v>3.2558825E8</v>
       </c>
       <c r="AA216" s="14" t="inlineStr"/>
       <c r="AB216" s="14" t="inlineStr"/>
       <c r="AC216" s="15" t="n">
-        <v>0.8841168805253546</v>
+        <v>0.9843997544958699</v>
       </c>
       <c r="AD216" s="15" t="inlineStr"/>
       <c r="AE216" s="14" t="n">
-        <v>3.832811E7</v>
+        <v>5159750.0</v>
       </c>
       <c r="AF216" s="14" t="inlineStr"/>
       <c r="AG216" s="14" t="inlineStr"/>
@@ -13230,23 +13230,23 @@
       <c r="U217" s="14" t="inlineStr"/>
       <c r="V217" s="14" t="inlineStr"/>
       <c r="W217" s="14" t="n">
-        <v>1.9270962E8</v>
+        <v>2.2587798E8</v>
       </c>
       <c r="X217" s="14" t="n">
         <v>3.316836E7</v>
       </c>
       <c r="Y217" s="14" t="inlineStr"/>
       <c r="Z217" s="14" t="n">
-        <v>2.2587798E8</v>
+        <v>2.5904634E8</v>
       </c>
       <c r="AA217" s="14" t="inlineStr"/>
       <c r="AB217" s="14" t="inlineStr"/>
       <c r="AC217" s="15" t="n">
-        <v>0.8555984090909091</v>
+        <v>0.9812361363636364</v>
       </c>
       <c r="AD217" s="15" t="inlineStr"/>
       <c r="AE217" s="14" t="n">
-        <v>3.812202E7</v>
+        <v>4953660.0</v>
       </c>
       <c r="AF217" s="14" t="inlineStr"/>
       <c r="AG217" s="14" t="inlineStr"/>
@@ -13407,10 +13407,10 @@
       <c r="U220" s="14" t="inlineStr"/>
       <c r="V220" s="14" t="inlineStr"/>
       <c r="W220" s="14" t="n">
-        <v>5.34431E8</v>
+        <v>6.44264E8</v>
       </c>
       <c r="X220" s="14" t="n">
-        <v>1.09833E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y220" s="14" t="inlineStr"/>
       <c r="Z220" s="14" t="n">
@@ -13464,10 +13464,10 @@
       <c r="U221" s="14" t="inlineStr"/>
       <c r="V221" s="14" t="inlineStr"/>
       <c r="W221" s="14" t="n">
-        <v>5.11E7</v>
+        <v>6.181E7</v>
       </c>
       <c r="X221" s="14" t="n">
-        <v>1.071E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y221" s="14" t="inlineStr"/>
       <c r="Z221" s="14" t="n">
@@ -13565,10 +13565,10 @@
       <c r="U223" s="14" t="inlineStr"/>
       <c r="V223" s="14" t="inlineStr"/>
       <c r="W223" s="14" t="n">
-        <v>4.83331E8</v>
+        <v>5.82454E8</v>
       </c>
       <c r="X223" s="14" t="n">
-        <v>9.9123E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y223" s="14" t="inlineStr"/>
       <c r="Z223" s="14" t="n">
@@ -13628,10 +13628,10 @@
       <c r="U224" s="14" t="inlineStr"/>
       <c r="V224" s="14" t="inlineStr"/>
       <c r="W224" s="14" t="n">
-        <v>5.215494289E9</v>
+        <v>5.981030439E9</v>
       </c>
       <c r="X224" s="14" t="n">
-        <v>7.6553615E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y224" s="14" t="inlineStr"/>
       <c r="Z224" s="14" t="n">
@@ -13685,10 +13685,10 @@
       <c r="U225" s="14" t="inlineStr"/>
       <c r="V225" s="14" t="inlineStr"/>
       <c r="W225" s="14" t="n">
-        <v>3.641050913E9</v>
+        <v>4.406587063E9</v>
       </c>
       <c r="X225" s="14" t="n">
-        <v>7.6553615E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y225" s="14" t="inlineStr"/>
       <c r="Z225" s="14" t="n">
@@ -13862,23 +13862,23 @@
       <c r="U228" s="25" t="inlineStr"/>
       <c r="V228" s="25" t="inlineStr"/>
       <c r="W228" s="25" t="n">
-        <v>2.551189645E9</v>
+        <v>2.97538798E9</v>
       </c>
       <c r="X228" s="25" t="n">
-        <v>4.24198335E8</v>
+        <v>7.341E7</v>
       </c>
       <c r="Y228" s="25" t="inlineStr"/>
       <c r="Z228" s="25" t="n">
-        <v>2.97538798E9</v>
+        <v>3.04879798E9</v>
       </c>
       <c r="AA228" s="25" t="inlineStr"/>
       <c r="AB228" s="25" t="inlineStr"/>
       <c r="AC228" s="26" t="n">
-        <v>0.5260801811389397</v>
+        <v>0.5390598484485487</v>
       </c>
       <c r="AD228" s="26" t="inlineStr"/>
       <c r="AE228" s="25" t="n">
-        <v>2.68038102E9</v>
+        <v>2.60697102E9</v>
       </c>
       <c r="AF228" s="25" t="inlineStr"/>
       <c r="AG228" s="25" t="inlineStr"/>
@@ -13925,23 +13925,23 @@
       <c r="U229" s="14" t="inlineStr"/>
       <c r="V229" s="14" t="inlineStr"/>
       <c r="W229" s="14" t="n">
-        <v>1.760022116E9</v>
+        <v>2.088338999E9</v>
       </c>
       <c r="X229" s="14" t="n">
-        <v>3.28316883E8</v>
+        <v>6.35E7</v>
       </c>
       <c r="Y229" s="14" t="inlineStr"/>
       <c r="Z229" s="14" t="n">
-        <v>2.088338999E9</v>
+        <v>2.151838999E9</v>
       </c>
       <c r="AA229" s="14" t="inlineStr"/>
       <c r="AB229" s="14" t="inlineStr"/>
       <c r="AC229" s="15" t="n">
-        <v>0.537586873631474</v>
+        <v>0.5539332457922893</v>
       </c>
       <c r="AD229" s="15" t="inlineStr"/>
       <c r="AE229" s="14" t="n">
-        <v>1.796315001E9</v>
+        <v>1.732815001E9</v>
       </c>
       <c r="AF229" s="14" t="inlineStr"/>
       <c r="AG229" s="14" t="inlineStr"/>
@@ -13988,23 +13988,23 @@
       <c r="U230" s="14" t="inlineStr"/>
       <c r="V230" s="14" t="inlineStr"/>
       <c r="W230" s="14" t="n">
-        <v>4.13618356E8</v>
+        <v>4.83128803E8</v>
       </c>
       <c r="X230" s="14" t="n">
-        <v>6.9510447E7</v>
+        <v>6.35E7</v>
       </c>
       <c r="Y230" s="14" t="inlineStr"/>
       <c r="Z230" s="14" t="n">
-        <v>4.83128803E8</v>
+        <v>5.46628803E8</v>
       </c>
       <c r="AA230" s="14" t="inlineStr"/>
       <c r="AB230" s="14" t="inlineStr"/>
       <c r="AC230" s="15" t="n">
-        <v>0.6575712866314513</v>
+        <v>0.7439991221109624</v>
       </c>
       <c r="AD230" s="15" t="inlineStr"/>
       <c r="AE230" s="14" t="n">
-        <v>2.51588197E8</v>
+        <v>1.88088197E8</v>
       </c>
       <c r="AF230" s="14" t="inlineStr"/>
       <c r="AG230" s="14" t="inlineStr"/>
@@ -14045,23 +14045,23 @@
       <c r="U231" s="14" t="inlineStr"/>
       <c r="V231" s="14" t="inlineStr"/>
       <c r="W231" s="14" t="n">
-        <v>3.845E8</v>
+        <v>4.48E8</v>
       </c>
       <c r="X231" s="14" t="n">
         <v>6.35E7</v>
       </c>
       <c r="Y231" s="14" t="inlineStr"/>
       <c r="Z231" s="14" t="n">
-        <v>4.48E8</v>
+        <v>5.115E8</v>
       </c>
       <c r="AA231" s="14" t="inlineStr"/>
       <c r="AB231" s="14" t="inlineStr"/>
       <c r="AC231" s="15" t="n">
-        <v>0.6588235294117647</v>
+        <v>0.7522058823529412</v>
       </c>
       <c r="AD231" s="15" t="inlineStr"/>
       <c r="AE231" s="14" t="n">
-        <v>2.32E8</v>
+        <v>1.685E8</v>
       </c>
       <c r="AF231" s="14" t="inlineStr"/>
       <c r="AG231" s="14" t="inlineStr"/>
@@ -14102,10 +14102,10 @@
       <c r="U232" s="14" t="inlineStr"/>
       <c r="V232" s="14" t="inlineStr"/>
       <c r="W232" s="14" t="n">
-        <v>2076300.0</v>
+        <v>2419200.0</v>
       </c>
       <c r="X232" s="14" t="n">
-        <v>342900.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y232" s="14" t="inlineStr"/>
       <c r="Z232" s="14" t="n">
@@ -14159,10 +14159,10 @@
       <c r="U233" s="14" t="inlineStr"/>
       <c r="V233" s="14" t="inlineStr"/>
       <c r="W233" s="14" t="n">
-        <v>2.7042056E7</v>
+        <v>3.2709603E7</v>
       </c>
       <c r="X233" s="14" t="n">
-        <v>5667547.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y233" s="14" t="inlineStr"/>
       <c r="Z233" s="14" t="n">
@@ -14222,10 +14222,10 @@
       <c r="U234" s="14" t="inlineStr"/>
       <c r="V234" s="14" t="inlineStr"/>
       <c r="W234" s="14" t="n">
-        <v>4157000.0</v>
+        <v>5144000.0</v>
       </c>
       <c r="X234" s="14" t="n">
-        <v>987000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y234" s="14" t="inlineStr"/>
       <c r="Z234" s="14" t="n">
@@ -14279,10 +14279,10 @@
       <c r="U235" s="14" t="inlineStr"/>
       <c r="V235" s="14" t="inlineStr"/>
       <c r="W235" s="14" t="n">
-        <v>2137000.0</v>
+        <v>2720000.0</v>
       </c>
       <c r="X235" s="14" t="n">
-        <v>583000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y235" s="14" t="inlineStr"/>
       <c r="Z235" s="14" t="n">
@@ -14336,10 +14336,10 @@
       <c r="U236" s="14" t="inlineStr"/>
       <c r="V236" s="14" t="inlineStr"/>
       <c r="W236" s="14" t="n">
-        <v>2020000.0</v>
+        <v>2424000.0</v>
       </c>
       <c r="X236" s="14" t="n">
-        <v>404000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y236" s="14" t="inlineStr"/>
       <c r="Z236" s="14" t="n">
@@ -14399,10 +14399,10 @@
       <c r="U237" s="14" t="inlineStr"/>
       <c r="V237" s="14" t="inlineStr"/>
       <c r="W237" s="14" t="n">
-        <v>8622580.0</v>
+        <v>1.280558E7</v>
       </c>
       <c r="X237" s="14" t="n">
-        <v>4183000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y237" s="14" t="inlineStr"/>
       <c r="Z237" s="14" t="n">
@@ -14456,10 +14456,10 @@
       <c r="U238" s="14" t="inlineStr"/>
       <c r="V238" s="14" t="inlineStr"/>
       <c r="W238" s="14" t="n">
-        <v>8622580.0</v>
+        <v>1.280558E7</v>
       </c>
       <c r="X238" s="14" t="n">
-        <v>4183000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y238" s="14" t="inlineStr"/>
       <c r="Z238" s="14" t="n">
@@ -14639,10 +14639,10 @@
       <c r="U241" s="14" t="inlineStr"/>
       <c r="V241" s="14" t="inlineStr"/>
       <c r="W241" s="14" t="n">
-        <v>1.33163418E9</v>
+        <v>1.585270616E9</v>
       </c>
       <c r="X241" s="14" t="n">
-        <v>2.53636436E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y241" s="14" t="inlineStr"/>
       <c r="Z241" s="14" t="n">
@@ -14696,10 +14696,10 @@
       <c r="U242" s="14" t="inlineStr"/>
       <c r="V242" s="14" t="inlineStr"/>
       <c r="W242" s="14" t="n">
-        <v>2.4455968E8</v>
+        <v>2.85881376E8</v>
       </c>
       <c r="X242" s="14" t="n">
-        <v>4.1321696E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y242" s="14" t="inlineStr"/>
       <c r="Z242" s="14" t="n">
@@ -14753,10 +14753,10 @@
       <c r="U243" s="14" t="inlineStr"/>
       <c r="V243" s="14" t="inlineStr"/>
       <c r="W243" s="14" t="n">
-        <v>5.597624E7</v>
+        <v>6.5444768E7</v>
       </c>
       <c r="X243" s="14" t="n">
-        <v>9468528.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y243" s="14" t="inlineStr"/>
       <c r="Z243" s="14" t="n">
@@ -14810,10 +14810,10 @@
       <c r="U244" s="14" t="inlineStr"/>
       <c r="V244" s="14" t="inlineStr"/>
       <c r="W244" s="14" t="n">
-        <v>8.129932E7</v>
+        <v>9.5029104E7</v>
       </c>
       <c r="X244" s="14" t="n">
-        <v>1.3729784E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y244" s="14" t="inlineStr"/>
       <c r="Z244" s="14" t="n">
@@ -14867,10 +14867,10 @@
       <c r="U245" s="14" t="inlineStr"/>
       <c r="V245" s="14" t="inlineStr"/>
       <c r="W245" s="14" t="n">
-        <v>2.736644E7</v>
+        <v>3.1996368E7</v>
       </c>
       <c r="X245" s="14" t="n">
-        <v>4629928.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y245" s="14" t="inlineStr"/>
       <c r="Z245" s="14" t="n">
@@ -14924,10 +14924,10 @@
       <c r="U246" s="14" t="inlineStr"/>
       <c r="V246" s="14" t="inlineStr"/>
       <c r="W246" s="14" t="n">
-        <v>9.224325E8</v>
+        <v>1.106919E9</v>
       </c>
       <c r="X246" s="14" t="n">
-        <v>1.844865E8</v>
+        <v>0.0</v>
       </c>
       <c r="Y246" s="14" t="inlineStr"/>
       <c r="Z246" s="14" t="n">
@@ -14987,10 +14987,10 @@
       <c r="U247" s="14" t="inlineStr"/>
       <c r="V247" s="14" t="inlineStr"/>
       <c r="W247" s="14" t="n">
-        <v>3.80681131E8</v>
+        <v>4.32620013E8</v>
       </c>
       <c r="X247" s="14" t="n">
-        <v>5.1938882E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y247" s="14" t="inlineStr"/>
       <c r="Z247" s="14" t="n">
@@ -15094,10 +15094,10 @@
       <c r="U249" s="14" t="inlineStr"/>
       <c r="V249" s="14" t="inlineStr"/>
       <c r="W249" s="14" t="n">
-        <v>2.73406741E8</v>
+        <v>3.10883859E8</v>
       </c>
       <c r="X249" s="14" t="n">
-        <v>3.7477118E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y249" s="14" t="inlineStr"/>
       <c r="Z249" s="14" t="n">
@@ -15151,10 +15151,10 @@
       <c r="U250" s="14" t="inlineStr"/>
       <c r="V250" s="14" t="inlineStr"/>
       <c r="W250" s="14" t="n">
-        <v>2.73406741E8</v>
+        <v>3.10883859E8</v>
       </c>
       <c r="X250" s="14" t="n">
-        <v>3.7477118E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y250" s="14" t="inlineStr"/>
       <c r="Z250" s="14" t="n">
@@ -15214,10 +15214,10 @@
       <c r="U251" s="14" t="inlineStr"/>
       <c r="V251" s="14" t="inlineStr"/>
       <c r="W251" s="14" t="n">
-        <v>4161834.0</v>
+        <v>4425348.0</v>
       </c>
       <c r="X251" s="14" t="n">
-        <v>263514.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y251" s="14" t="inlineStr"/>
       <c r="Z251" s="14" t="n">
@@ -15271,10 +15271,10 @@
       <c r="U252" s="14" t="inlineStr"/>
       <c r="V252" s="14" t="inlineStr"/>
       <c r="W252" s="14" t="n">
-        <v>4161834.0</v>
+        <v>4425348.0</v>
       </c>
       <c r="X252" s="14" t="n">
-        <v>263514.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y252" s="14" t="inlineStr"/>
       <c r="Z252" s="14" t="n">
@@ -15334,10 +15334,10 @@
       <c r="U253" s="14" t="inlineStr"/>
       <c r="V253" s="14" t="inlineStr"/>
       <c r="W253" s="14" t="n">
-        <v>2.13328E7</v>
+        <v>2.48451E7</v>
       </c>
       <c r="X253" s="14" t="n">
-        <v>3512300.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y253" s="14" t="inlineStr"/>
       <c r="Z253" s="14" t="n">
@@ -15391,10 +15391,10 @@
       <c r="U254" s="14" t="inlineStr"/>
       <c r="V254" s="14" t="inlineStr"/>
       <c r="W254" s="14" t="n">
-        <v>2.13328E7</v>
+        <v>2.48451E7</v>
       </c>
       <c r="X254" s="14" t="n">
-        <v>3512300.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y254" s="14" t="inlineStr"/>
       <c r="Z254" s="14" t="n">
@@ -15454,10 +15454,10 @@
       <c r="U255" s="14" t="inlineStr"/>
       <c r="V255" s="14" t="inlineStr"/>
       <c r="W255" s="14" t="n">
-        <v>8.1779756E7</v>
+        <v>9.2465706E7</v>
       </c>
       <c r="X255" s="14" t="n">
-        <v>1.068595E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y255" s="14" t="inlineStr"/>
       <c r="Z255" s="14" t="n">
@@ -15511,10 +15511,10 @@
       <c r="U256" s="14" t="inlineStr"/>
       <c r="V256" s="14" t="inlineStr"/>
       <c r="W256" s="14" t="n">
-        <v>5.607995E7</v>
+        <v>6.58569E7</v>
       </c>
       <c r="X256" s="14" t="n">
-        <v>9776950.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y256" s="14" t="inlineStr"/>
       <c r="Z256" s="14" t="n">
@@ -15568,10 +15568,10 @@
       <c r="U257" s="14" t="inlineStr"/>
       <c r="V257" s="14" t="inlineStr"/>
       <c r="W257" s="14" t="n">
-        <v>2.5699806E7</v>
+        <v>2.6608806E7</v>
       </c>
       <c r="X257" s="14" t="n">
-        <v>909000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y257" s="14" t="inlineStr"/>
       <c r="Z257" s="14" t="n">
@@ -15631,10 +15631,10 @@
       <c r="U258" s="14" t="inlineStr"/>
       <c r="V258" s="14" t="inlineStr"/>
       <c r="W258" s="14" t="n">
-        <v>3.51036398E8</v>
+        <v>3.84588968E8</v>
       </c>
       <c r="X258" s="14" t="n">
-        <v>3.355257E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y258" s="14" t="inlineStr"/>
       <c r="Z258" s="14" t="n">
@@ -15991,10 +15991,10 @@
       <c r="U264" s="14" t="inlineStr"/>
       <c r="V264" s="14" t="inlineStr"/>
       <c r="W264" s="14" t="n">
-        <v>9.0095326E7</v>
+        <v>1.10331326E8</v>
       </c>
       <c r="X264" s="14" t="n">
-        <v>2.0236E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y264" s="14" t="inlineStr"/>
       <c r="Z264" s="14" t="n">
@@ -16048,10 +16048,10 @@
       <c r="U265" s="14" t="inlineStr"/>
       <c r="V265" s="14" t="inlineStr"/>
       <c r="W265" s="14" t="n">
-        <v>1.5716622E7</v>
+        <v>1.6931622E7</v>
       </c>
       <c r="X265" s="14" t="n">
-        <v>1215000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y265" s="14" t="inlineStr"/>
       <c r="Z265" s="14" t="n">
@@ -16105,10 +16105,10 @@
       <c r="U266" s="14" t="inlineStr"/>
       <c r="V266" s="14" t="inlineStr"/>
       <c r="W266" s="14" t="n">
-        <v>1.0101299E7</v>
+        <v>1.1156299E7</v>
       </c>
       <c r="X266" s="14" t="n">
-        <v>1055000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y266" s="14" t="inlineStr"/>
       <c r="Z266" s="14" t="n">
@@ -16162,10 +16162,10 @@
       <c r="U267" s="14" t="inlineStr"/>
       <c r="V267" s="14" t="inlineStr"/>
       <c r="W267" s="14" t="n">
-        <v>1.155E7</v>
+        <v>2.5327E7</v>
       </c>
       <c r="X267" s="14" t="n">
-        <v>1.3777E7</v>
+        <v>0.0</v>
       </c>
       <c r="Y267" s="14" t="inlineStr"/>
       <c r="Z267" s="14" t="n">
@@ -16662,10 +16662,10 @@
       <c r="U276" s="14" t="inlineStr"/>
       <c r="V276" s="14" t="inlineStr"/>
       <c r="W276" s="14" t="n">
-        <v>1.1095E7</v>
+        <v>1.5284E7</v>
       </c>
       <c r="X276" s="14" t="n">
-        <v>4189000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y276" s="14" t="inlineStr"/>
       <c r="Z276" s="14" t="n">
@@ -16839,10 +16839,10 @@
       <c r="U279" s="14" t="inlineStr"/>
       <c r="V279" s="14" t="inlineStr"/>
       <c r="W279" s="14" t="n">
-        <v>8.3881357E7</v>
+        <v>8.8386927E7</v>
       </c>
       <c r="X279" s="14" t="n">
-        <v>4505570.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y279" s="14" t="inlineStr"/>
       <c r="Z279" s="14" t="n">
@@ -17067,10 +17067,10 @@
       <c r="U283" s="14" t="inlineStr"/>
       <c r="V283" s="14" t="inlineStr"/>
       <c r="W283" s="14" t="n">
-        <v>6.3191077E7</v>
+        <v>6.6116077E7</v>
       </c>
       <c r="X283" s="14" t="n">
-        <v>2925000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y283" s="14" t="inlineStr"/>
       <c r="Z283" s="14" t="n">
@@ -17124,10 +17124,10 @@
       <c r="U284" s="14" t="inlineStr"/>
       <c r="V284" s="14" t="inlineStr"/>
       <c r="W284" s="14" t="n">
-        <v>2027000.0</v>
+        <v>2177000.0</v>
       </c>
       <c r="X284" s="14" t="n">
-        <v>150000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y284" s="14" t="inlineStr"/>
       <c r="Z284" s="14" t="n">
@@ -17181,10 +17181,10 @@
       <c r="U285" s="14" t="inlineStr"/>
       <c r="V285" s="14" t="inlineStr"/>
       <c r="W285" s="14" t="n">
-        <v>4686025.0</v>
+        <v>4737535.0</v>
       </c>
       <c r="X285" s="14" t="n">
-        <v>51510.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y285" s="14" t="inlineStr"/>
       <c r="Z285" s="14" t="n">
@@ -17352,10 +17352,10 @@
       <c r="U288" s="14" t="inlineStr"/>
       <c r="V288" s="14" t="inlineStr"/>
       <c r="W288" s="14" t="n">
-        <v>2597953.0</v>
+        <v>3707013.0</v>
       </c>
       <c r="X288" s="14" t="n">
-        <v>1109060.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y288" s="14" t="inlineStr"/>
       <c r="Z288" s="14" t="n">
@@ -17523,10 +17523,10 @@
       <c r="U291" s="14" t="inlineStr"/>
       <c r="V291" s="14" t="inlineStr"/>
       <c r="W291" s="14" t="n">
-        <v>0.0</v>
+        <v>270000.0</v>
       </c>
       <c r="X291" s="14" t="n">
-        <v>270000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y291" s="14" t="inlineStr"/>
       <c r="Z291" s="14" t="n">
@@ -17586,10 +17586,10 @@
       <c r="U292" s="14" t="inlineStr"/>
       <c r="V292" s="14" t="inlineStr"/>
       <c r="W292" s="14" t="n">
-        <v>5.2605E7</v>
+        <v>6.1416E7</v>
       </c>
       <c r="X292" s="14" t="n">
-        <v>8811000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y292" s="14" t="inlineStr"/>
       <c r="Z292" s="14" t="n">
@@ -17757,10 +17757,10 @@
       <c r="U295" s="14" t="inlineStr"/>
       <c r="V295" s="14" t="inlineStr"/>
       <c r="W295" s="14" t="n">
-        <v>1965000.0</v>
+        <v>1.0776E7</v>
       </c>
       <c r="X295" s="14" t="n">
-        <v>8811000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y295" s="14" t="inlineStr"/>
       <c r="Z295" s="14" t="n">
@@ -17820,23 +17820,23 @@
       <c r="U296" s="14" t="inlineStr"/>
       <c r="V296" s="14" t="inlineStr"/>
       <c r="W296" s="14" t="n">
-        <v>5.945E7</v>
+        <v>6.984E7</v>
       </c>
       <c r="X296" s="14" t="n">
-        <v>1.039E7</v>
+        <v>9910000.0</v>
       </c>
       <c r="Y296" s="14" t="inlineStr"/>
       <c r="Z296" s="14" t="n">
-        <v>6.984E7</v>
+        <v>7.975E7</v>
       </c>
       <c r="AA296" s="14" t="inlineStr"/>
       <c r="AB296" s="14" t="inlineStr"/>
       <c r="AC296" s="15" t="n">
-        <v>0.5283704039945529</v>
+        <v>0.6033439249508247</v>
       </c>
       <c r="AD296" s="15" t="inlineStr"/>
       <c r="AE296" s="14" t="n">
-        <v>6.234E7</v>
+        <v>5.243E7</v>
       </c>
       <c r="AF296" s="14" t="inlineStr"/>
       <c r="AG296" s="14" t="inlineStr"/>
@@ -17883,23 +17883,23 @@
       <c r="U297" s="14" t="inlineStr"/>
       <c r="V297" s="14" t="inlineStr"/>
       <c r="W297" s="14" t="n">
-        <v>5.195E7</v>
+        <v>6.234E7</v>
       </c>
       <c r="X297" s="14" t="n">
-        <v>1.039E7</v>
+        <v>9910000.0</v>
       </c>
       <c r="Y297" s="14" t="inlineStr"/>
       <c r="Z297" s="14" t="n">
-        <v>6.234E7</v>
+        <v>7.225E7</v>
       </c>
       <c r="AA297" s="14" t="inlineStr"/>
       <c r="AB297" s="14" t="inlineStr"/>
       <c r="AC297" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5794834777029195</v>
       </c>
       <c r="AD297" s="15" t="inlineStr"/>
       <c r="AE297" s="14" t="n">
-        <v>6.234E7</v>
+        <v>5.243E7</v>
       </c>
       <c r="AF297" s="14" t="inlineStr"/>
       <c r="AG297" s="14" t="inlineStr"/>
@@ -17940,23 +17940,23 @@
       <c r="U298" s="14" t="inlineStr"/>
       <c r="V298" s="14" t="inlineStr"/>
       <c r="W298" s="14" t="n">
-        <v>1.275E7</v>
+        <v>1.53E7</v>
       </c>
       <c r="X298" s="14" t="n">
         <v>2550000.0</v>
       </c>
       <c r="Y298" s="14" t="inlineStr"/>
       <c r="Z298" s="14" t="n">
-        <v>1.53E7</v>
+        <v>1.785E7</v>
       </c>
       <c r="AA298" s="14" t="inlineStr"/>
       <c r="AB298" s="14" t="inlineStr"/>
       <c r="AC298" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD298" s="15" t="inlineStr"/>
       <c r="AE298" s="14" t="n">
-        <v>1.53E7</v>
+        <v>1.275E7</v>
       </c>
       <c r="AF298" s="14" t="inlineStr"/>
       <c r="AG298" s="14" t="inlineStr"/>
@@ -17997,23 +17997,23 @@
       <c r="U299" s="14" t="inlineStr"/>
       <c r="V299" s="14" t="inlineStr"/>
       <c r="W299" s="14" t="n">
-        <v>1.24E7</v>
+        <v>1.488E7</v>
       </c>
       <c r="X299" s="14" t="n">
         <v>2480000.0</v>
       </c>
       <c r="Y299" s="14" t="inlineStr"/>
       <c r="Z299" s="14" t="n">
-        <v>1.488E7</v>
+        <v>1.736E7</v>
       </c>
       <c r="AA299" s="14" t="inlineStr"/>
       <c r="AB299" s="14" t="inlineStr"/>
       <c r="AC299" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD299" s="15" t="inlineStr"/>
       <c r="AE299" s="14" t="n">
-        <v>1.488E7</v>
+        <v>1.24E7</v>
       </c>
       <c r="AF299" s="14" t="inlineStr"/>
       <c r="AG299" s="14" t="inlineStr"/>
@@ -18054,23 +18054,23 @@
       <c r="U300" s="14" t="inlineStr"/>
       <c r="V300" s="14" t="inlineStr"/>
       <c r="W300" s="14" t="n">
-        <v>6150000.0</v>
+        <v>7380000.0</v>
       </c>
       <c r="X300" s="14" t="n">
         <v>1230000.0</v>
       </c>
       <c r="Y300" s="14" t="inlineStr"/>
       <c r="Z300" s="14" t="n">
-        <v>7380000.0</v>
+        <v>8610000.0</v>
       </c>
       <c r="AA300" s="14" t="inlineStr"/>
       <c r="AB300" s="14" t="inlineStr"/>
       <c r="AC300" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD300" s="15" t="inlineStr"/>
       <c r="AE300" s="14" t="n">
-        <v>7380000.0</v>
+        <v>6150000.0</v>
       </c>
       <c r="AF300" s="14" t="inlineStr"/>
       <c r="AG300" s="14" t="inlineStr"/>
@@ -18111,23 +18111,23 @@
       <c r="U301" s="14" t="inlineStr"/>
       <c r="V301" s="14" t="inlineStr"/>
       <c r="W301" s="14" t="n">
-        <v>5350000.0</v>
+        <v>6420000.0</v>
       </c>
       <c r="X301" s="14" t="n">
         <v>1070000.0</v>
       </c>
       <c r="Y301" s="14" t="inlineStr"/>
       <c r="Z301" s="14" t="n">
-        <v>6420000.0</v>
+        <v>7490000.0</v>
       </c>
       <c r="AA301" s="14" t="inlineStr"/>
       <c r="AB301" s="14" t="inlineStr"/>
       <c r="AC301" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD301" s="15" t="inlineStr"/>
       <c r="AE301" s="14" t="n">
-        <v>6420000.0</v>
+        <v>5350000.0</v>
       </c>
       <c r="AF301" s="14" t="inlineStr"/>
       <c r="AG301" s="14" t="inlineStr"/>
@@ -18212,23 +18212,23 @@
       <c r="U303" s="14" t="inlineStr"/>
       <c r="V303" s="14" t="inlineStr"/>
       <c r="W303" s="14" t="n">
-        <v>1.2E7</v>
+        <v>1.44E7</v>
       </c>
       <c r="X303" s="14" t="n">
         <v>2400000.0</v>
       </c>
       <c r="Y303" s="14" t="inlineStr"/>
       <c r="Z303" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.68E7</v>
       </c>
       <c r="AA303" s="14" t="inlineStr"/>
       <c r="AB303" s="14" t="inlineStr"/>
       <c r="AC303" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5833333333333334</v>
       </c>
       <c r="AD303" s="15" t="inlineStr"/>
       <c r="AE303" s="14" t="n">
-        <v>1.44E7</v>
+        <v>1.2E7</v>
       </c>
       <c r="AF303" s="14" t="inlineStr"/>
       <c r="AG303" s="14" t="inlineStr"/>
@@ -18269,10 +18269,10 @@
       <c r="U304" s="14" t="inlineStr"/>
       <c r="V304" s="14" t="inlineStr"/>
       <c r="W304" s="14" t="n">
-        <v>1500000.0</v>
+        <v>1800000.0</v>
       </c>
       <c r="X304" s="14" t="n">
-        <v>300000.0</v>
+        <v>0.0</v>
       </c>
       <c r="Y304" s="14" t="inlineStr"/>
       <c r="Z304" s="14" t="n">
@@ -18326,23 +18326,23 @@
       <c r="U305" s="14" t="inlineStr"/>
       <c r="V305" s="14" t="inlineStr"/>
       <c r="W305" s="14" t="n">
-        <v>1800000.0</v>
+        <v>2160000.0</v>
       </c>
       <c r="X305" s="14" t="n">
-        <v>360000.0</v>
+        <v>180000.0</v>
       </c>
       <c r="Y305" s="14" t="inlineStr"/>
       <c r="Z305" s="14" t="n">
-        <v>2160000.0</v>
+        <v>2340000.0</v>
       </c>
       <c r="AA305" s="14" t="inlineStr"/>
       <c r="AB305" s="14" t="inlineStr"/>
       <c r="AC305" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="AD305" s="15" t="inlineStr"/>
       <c r="AE305" s="14" t="n">
-        <v>2160000.0</v>
+        <v>1980000.0</v>
       </c>
       <c r="AF305" s="14" t="inlineStr"/>
       <c r="AG305" s="14" t="inlineStr"/>

</xml_diff>